<commit_message>
Strip Markdown from tracker cells and fix sentence endings
</commit_message>
<xml_diff>
--- a/tracker/WeConnect-QA-Bug-Tracker.xlsx
+++ b/tracker/WeConnect-QA-Bug-Tracker.xlsx
@@ -776,7 +776,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Run: node verify/run.mjs --only &lt;Bug ID&gt;   — no installation, read-only by default. The Re-check Command column gives the exact line.</t>
+          <t>Run: node verify/run.mjs --only &lt;Bug ID&gt; — no installation, read-only by default. The Re-check Command column gives the exact line.</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="J2" s="7" t="inlineStr">
         <is>
-          <t>HTTP 200. **10 of 10 records returned were wholly outside OC's permitted centres** — OC is permitted for 2 centres and received none of them. The records carry: `youth`, `youth_name`, `youth_stage`, `counselling_type`, `counselling_subtype`, `counselling_date`, `counselling_location`, `remarks`, `last_call_remarks`, `status`, `interested_course`, `batch`</t>
+          <t>HTTP 200. 10 of 10 records returned were wholly outside OC's permitted centres — OC is permitted for 2 centres and received none of them. The records carry: youth, youth_name, youth_stage, counselling_type, counselling_subtype, counselling_date, counselling_location, remarks, last_call_remarks, status, interested_course, batch.</t>
         </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>1. **Remove the `System Manager` bypass from handlers that return youth records.** A superuser role should not silently disable centre scoping on safeguarding-sensitive data; if an administrative override is genuinely required it should be explicit, narrow and audited. 2. **Remove the need for the role.** Persona accounts hold `System Manager` because the doctype permission model offers nothing else — see the permission-design finding. Until that is fixed, every endpoint guarded this way is open to every staff account. The originally recorded fix — "apply `permitted_centres` as a server-side filter" — would change nothing, because that filter is already present and already correct.</t>
+          <t>1. Remove the System Manager bypass from handlers that return youth records. A superuser role should not silently disable centre scoping on safeguarding-sensitive data; if an administrative override is genuinely required it should be explicit, narrow and audited. 2. Remove the need for the role. Persona accounts hold System Manager because the doctype permission model offers nothing else — see the permission-design finding. Until that is fixed, every endpoint guarded this way is open to every staff account. The originally recorded fix — "apply permitted_centres as a server-side filter" — would change nothing, because that filter is already present and already correct.</t>
         </is>
       </c>
       <c r="M2" s="7" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>A Skilling Batch was created owned by **QA North Centre**. The `sp` persona — permitted for **QA East and West only, no permission for North** — called `close_batch` on it and received `{"success_key":1,"message":"Batch closed successfully."}`. Ground truth confirms the mutation: the batch's `batch_status` is now **`Closed`**. A user closed a batch belonging to a centre they have no permission over.</t>
+          <t>A Skilling Batch was created owned by QA North Centre. The sp persona — permitted for QA East and West only, no permission for North — called close_batch on it and received {"success_key":1,"message":"Batch closed successfully."}. Ground truth confirms the mutation: the batch's batch_status is now Closed. A user closed a batch belonging to a centre they have no permission over.</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>check `location_lcf` against the caller's `permitted_centres` before closing, and remove `ignore_permissions=True` from the save. The same fix pattern applies across the class.</t>
+          <t>check location_lcf against the caller's permitted_centres before closing, and remove ignore_permissions=True from the save. The same fix pattern applies across the class.</t>
         </is>
       </c>
       <c r="M3" s="7" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>A Skilling Invoice was created for **QA North Centre**. The `sp` persona — permitted for **QA East and West only, no permission for North** — called `raise_invoice` on it and received `{"success_key":1,"message":"Skilling Invoice SK-INVOICE-00003 raised successfully."}`. Ground truth confirms the mutation: the invoice's `current_status` is now **`Raised`** and its `approval_status` is **`Verification Pending`** — it has entered the financial approval pipeline, moved there by a user with no permission over its centre. - **`prepare_tax_invoice` is breached the same way** — the same persona retrieved the North invoice's full tax-preparation details (`success_key:1`, invoice metadata returned), a financial data exposure across the boundary in addition to the write.</t>
+          <t>A Skilling Invoice was created for QA North Centre. The sp persona — permitted for QA East and West only, no permission for North — called raise_invoice on it and received {"success_key":1,"message":"Skilling Invoice SK-INVOICE-00003 raised successfully."}. Ground truth confirms the mutation: the invoice's current_status is now Raised and its approval_status is Verification Pending — it has entered the financial approval pipeline, moved there by a user with no permission over its centre. - prepare_tax_invoice is breached the same way — the same persona retrieved the North invoice's full tax-preparation details (success_key:1, invoice metadata returned), a financial data exposure across the boundary in addition to the write.</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>derive `center` from the caller's permitted scope; do not accept it as a parameter; remove `ignore_permissions=True`. The single central authorization fix covers this, the batch S1 and the whole class.</t>
+          <t>derive center from the caller's permitted scope; do not accept it as a parameter; remove ignore_permissions=True. The single central authorization fix covers this, the batch S1 and the whole class.</t>
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>See register</t>
+          <t>See register.</t>
         </is>
       </c>
       <c r="M5" s="7" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>HTTP 500 with a JSON body (1,705 chars) containing `exception`, `exc_type`, `_exc_source`, `exc`. The `exc` field carries a **full Python traceback including server filesystem paths**. `exc_type` is **`NameError`**.</t>
+          <t>HTTP 500 with a JSON body (1,705 chars) containing exception, exc_type, _exc_source, exc. The exc field carries a full Python traceback including server filesystem paths. exc_type is NameError.</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>disable client-facing traceback rendering in the deployed site config, and return 403 from this endpoint for roles without screening access. Then fix the `NameError`.</t>
+          <t>disable client-facing traceback rendering in the deployed site config, and return 403 from this endpoint for roles without screening access. Then fix the NameError.</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>- **Supersedes** the retracted clean result above. Found only after the scope checker was corrected to inspect the `data` envelope rather than the status string in `message`. Test used:** a record counts as an unambiguous violation only when it carries **no** centre the caller is permitted for. A record spanning several centres, one of which the caller owns, is excluded as arguable. Reproduced across every recorded query variant.</t>
+          <t>Supersedes the retracted clean result above. Found only after the scope checker was corrected to inspect the data envelope rather than the status string in message. Test used: a record counts as an unambiguous violation only when it carries no centre the caller is permitted for. A record spanning several centres, one of which the caller owns, is excluded as arguable. Reproduced across every recorded query variant.</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>1. For `approval_list` and `get_waiting_for_skilling_count`: **remove the `System Manager` early-return from the scope resolvers**, and fix the permission model so the role is not required (see the 45-site finding). Adding a filter would change nothing. The filter exists. 2. For `get_approvals`: confirm with the client whether the live account's `User Permission` rows matched its published `permitted_centres` at the time of observation, which would settle the dual-mechanism question. 3. Note that `dashboard.get_invoice_count` applies **no scoping at all** — `frappe.db.count("Skilling Invoice", {...})` with no centre filter — recorded separately.</t>
+          <t>1. For approval_list and get_waiting_for_skilling_count: remove the System Manager early-return from the scope resolvers, and fix the permission model so the role is not required (see the 45-site finding). Adding a filter would change nothing. The filter exists. 2. For get_approvals: confirm with the client whether the live account's User Permission rows matched its published permitted_centres at the time of observation, which would settle the dual-mechanism question. 3. Note that dashboard.get_invoice_count applies no scoping at all — frappe.db.count("Skilling Invoice", {...}) with no centre filter — recorded separately.</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
@@ -1532,7 +1532,7 @@
       <c r="H8" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as Skilling Partner.
-2. Call `/sp/invoicing/view-batch-invoice/prepare-invoice/:batchId/:installment/:centerName` and the equivalent `/sm/invoicing-management/...` route. once and note the resulting record.
+2. Call /sp/invoicing/view-batch-invoice/prepare-invoice/:batchId/:installment/:centerName and the equivalent /sm/invoicing-management/... route once and note the resulting record.
 3. Call it again with exactly the same payload.
 4. Check whether a second record or a second effect appeared.</t>
         </is>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>on page load, with no interaction whatsoever, the application issues `POST .../youth_skilling.api.invoice.prepare_tax_invoice?batch_id=&lt;batch&gt;&amp;installment=1&amp;center=&lt;centre&gt;`. Reproduced on both the Skilling Partner and Skilling Manager applications.</t>
+          <t>on page load, with no interaction whatsoever, the application issues POST .../youth_skilling.api.invoice.prepare_tax_invoice?batch_id=&lt;batch&gt;&amp;installment=1&amp;center=&lt;centre&gt;. Reproduced on both the Skilling Partner and Skilling Manager applications.</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
@@ -1636,17 +1636,17 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>the full sweep captures uncaught JavaScript exceptions. Five routes throw: | Persona | Route | Exception | |---|---|---| | FC | `/fc/badge-table` | `Cannot read properties of null (reading 'viewType')` | | FC | `/fc/batch-management/view-batch` | `Cannot read properties of null (reading 'batchId')` | | FC | `/fc/view-post-test` | `Cannot read properties of null (reading 'batch_id')` | | FC | `/fc/group-based-counselling/attendance` | `Cannot read properties of null (reading 'length')` | | SYC | `/group-based-counselling/attendance` | `Cannot read properties of null (reading 'length')` |</t>
+          <t>the full sweep captures uncaught JavaScript exceptions. Five routes throw:; Persona; Route; Exception; FC; /fc/badge-table; Cannot read properties of null (reading 'viewType'); FC; /fc/batch-management/view-batch; Cannot read properties of null (reading 'batchId'); FC; /fc/view-post-test; Cannot read properties of null (reading 'batch_id'); FC; /fc/group-based-counselling/attendance; Cannot read properties of null (reading 'length'); SYC; /group-based-counselling/attendance; Cannot read properties of null (reading 'length')</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>test-results-run1/sweep-route-sweep--fc-rout-c69cf--fc-badge-table-BadgeTable--fc-retry1/test-failed-1.png · test-results-run1/sweep-route-sweep--fc-rout-4948a-ement-view-batch-ViewBatch--fc/test-failed-1.png · test-results-run1/sweep-route-sweep--fc-rout-857ce-iew-post-test-ViewPostTest--fc/test-fa · evidence/validation-probe-results.json · suite/probes/validation-probe.mjs · re-check: node verify/run.mjs --only WC-</t>
+          <t>test-results-run1/sweep-route-sweep--fc-rout-c69cf--fc-badge-table-BadgeTable--fc-retry1/test-failed-1.png · test-results-run1/sweep-route-sweep--fc-rout-4948a-ement-view-batch-ViewBatch--fc/test-failed-1.png · test-results-run1/sweep-route-sweep--fc-rout-857ce-iew-post-test-ViewPostTest--fc/test-fa · evidence/validation-probe-results.json · suite/probes/validation-probe.mjs … (full detail in the findings register)</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>read identifiers from URL parameters rather than router state, and guard the state access (`location.state?.batchId`). The identifier is already in the URL for the `:batchId` routes, so the data needed is present. It is simply not being read from there.</t>
+          <t>read identifiers from URL parameters rather than router state, and guard the state access (location.state?.batchId). The identifier is already in the URL for the :batchId routes, so the data needed is present. It is simply not being read from there.</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>`GET {BACKEND}/api/method/youth_skilling.api.docs.swagger_spec` **with no Authorization header** returns HTTP 200 and the full specification.</t>
+          <t>GET {BACKEND}/api/method/youth_skilling.api.docs.swagger_spec with no Authorization header returns HTTP 200 and the full specification.</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>remove `allow_guest=True` from the three `swagger_spec` functions. The specifications remain available to authenticated staff, which is presumably the intent. This is a one-word change in three places.</t>
+          <t>remove allow_guest=True from the three swagger_spec functions. The specifications remain available to authenticated staff, which is presumably the intent. This is a one-word change in three places.</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
@@ -1820,7 +1820,7 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>| Fact | Value | |---|---| | WeConnect doctypes | 293 | | granting **only** `System Manager` | **178** | | granting **no role at all** | 115 | | granting any other role | **0** | | API endpoints passing `ignore_permissions=True` | 296 of 866 |</t>
+          <t>Fact; Value; WeConnect doctypes; 293; granting only System Manager; 178; granting no role at all; 115; granting any other role; 0; API endpoints passing ignore_permissions=True; 296 of 866.</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1901,7 +1901,7 @@
       <c r="H12" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as an authenticated staff account — any authenticated account is enough.
-2. Call `weconnect-backend-authentication`, `authentication/api/registration.py`, `create_user(email, first_name, last_name)`, decorated `@frappe.whitelist(methods=["POST"], allow_guest=True)`. with no special privileges.
+2. Call weconnect-backend-authentication, authentication/api/registration.py, create_user(email, first_name, last_name), decorated @frappe.whitelist(methods=["POST"], allow_guest=True) with no special privileges.
 3. Observe that the call is accepted rather than refused, and check whether anything changed.</t>
         </is>
       </c>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>An unauthenticated endpoint attempts to provision a System Manager account</t>
+          <t>An unauthenticated endpoint attempts to provision a System Manager account.</t>
         </is>
       </c>
       <c r="K12" s="7" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>(1) require an authenticated caller with an appropriate role — remove `allow_guest=True`; (2) do not grant `System Manager` on self-service creation — assign the least-privilege role the account needs; (3) if open registration is intended, separate "request an account" from "grant roles" so the two are never the same call.</t>
+          <t>(1) require an authenticated caller with an appropriate role — remove allow_guest=True; (2) do not grant System Manager on self-service creation — assign the least-privilege role the account needs; (3) if open registration is intended, separate "request an account" from "grant roles" so the two are never the same call.</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
@@ -1993,7 +1993,7 @@
       <c r="H13" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as Skilling Partner — any authenticated account is enough.
-2. Call `weconnect-backend-outreach`, `outreach/apis/registration/files.py`, `delete_file_by_url()`, `@frappe.whitelist(methods=["POST"])`. with no special privileges.
+2. Call weconnect-backend-outreach, outreach/apis/registration/files.py, delete_file_by_url(), @frappe.whitelist(methods=["POST"]) with no special privileges.
 3. Observe that the call is accepted rather than refused, and check whether anything changed.</t>
         </is>
       </c>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Of 214 mutating endpoints, **39 bypass permissions and contain no authorization check of any kind.** Of those, **35 also perform a direct write** — they are not merely unguarded reads mislabelled, they change data. The remaining 4 route through an approval or do not write.</t>
+          <t>Of 214 mutating endpoints, 39 bypass permissions and contain no authorization check of any kind. Of those, 35 also perform a direct write — they are not merely unguarded reads mislabelled, they change data. The remaining 4 route through an approval or do not write.</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>Financial endpoints share the confirmed cross-centre write gap</t>
+          <t>Financial endpoints share the confirmed cross-centre write gap.</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>derive `center` from the caller's permitted scope rather than accepting it as a parameter, and remove `ignore_permissions=True`. Same pattern as the close_batch fix.</t>
+          <t>derive center from the caller's permitted scope rather than accepting it as a parameter, and remove ignore_permissions=True. Same pattern as the close_batch fix.</t>
         </is>
       </c>
       <c r="M15" s="7" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>A valid Enquiry Form was created and its status change attempted through the API; the endpoint returned HTTP 500 `UnboundLocalError`. Confirmed against source.</t>
+          <t>A valid Enquiry Form was created and its status change attempted through the API; the endpoint returned HTTP 500 UnboundLocalError. Confirmed against source.</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>`ids = json.loads(ids)`. A one-word correction, and a test that calls the endpoint would have caught it — which is the point of this phase.</t>
+          <t>ids = json.loads(ids). A one-word correction, and a test that calls the endpoint would have caught it — which is the point of this phase.</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Systemic: data scoping is disabled for `System Manager` in application code, at 45 sites, while the platform forces that role onto every staff account</t>
+          <t>Systemic: data scoping is disabled for System Manager in application code, at 45 sites, while the platform forces that role onto every staff account</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>The Outreach Coordinator credential reports `permitted_centres = ["Kukatpally", "Bhawani Peth"]`, yet `GET /api/resource/Role Profile` and `GET /api/resource/User` both return **200** — reads only a System Manager obtains. That elevation is what produced the counselling S1: 10 of 10 youth counselling records returned from centres the account has no permission for.</t>
+          <t>The Outreach Coordinator credential reports permitted_centres = ["Kukatpally", "Bhawani Peth"], yet GET /api/resource/Role Profile and GET /api/resource/User both return 200 — reads only a System Manager obtains. That elevation is what produced the counselling S1: 10 of 10 youth counselling records returned from centres the account has no permission for.</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>1. **Remove the role check from data-scoping paths.** Scoping should not be conditional on a role. Where a genuine administrative override is needed, make it explicit, narrow and audited — not a blanket `pass` on youth records. 2. **Remove the need for the role**, by giving each persona role real doctype permissions. Until that lands, fixing (1) alone will lock staff out, so the two must ship together. 3. Add a test asserting that a non-administrative account cannot read a record outside its permitted centres, for each list endpoint.</t>
+          <t>1. Remove the role check from data-scoping paths. Scoping should not be conditional on a role. Where a genuine administrative override is needed, make it explicit, narrow and audited — not a blanket pass on youth records. 2. Remove the need for the role, by giving each persona role real doctype permissions. Until that lands, fixing (1) alone will lock staff out, so the two must ship together. 3. Add a test asserting that a non-administrative account cannot read a record outside its permitted centres, for each list endpoint.</t>
         </is>
       </c>
       <c r="M17" s="7" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>Called on the isolated instance as `sp` — the **Skilling Partner** persona, which represents an external training provider and is the lowest-trust account in the system — the endpoint returned **HTTP 200** and reached its own logic, failing only with `"LCF Google Sheet ID is not set in Google Integration Settings."` That failure is downstream of where a permission check belongs. The same result for `fc`. **No caller was refused.**</t>
+          <t>Called on the isolated instance as sp — the Skilling Partner persona, which represents an external training provider and is the lowest-trust account in the system — the endpoint returned HTTP 200 and reached its own logic, failing only with "LCF Google Sheet ID is not set in Google Integration Settings." That failure is downstream of where a permission check belongs. The same result for fc. No caller was refused.</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>404; widget shows "Data not available."</t>
+          <t>404; widget shows "Data not available.".</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>the widget calls an endpoint that is not present on the deployed build. Either restore `centre_head.api.target.main_dashboard.main_target` or remove the card that calls it. Either way the frontend should render an explicit empty state rather than the literal string shown today; the broken wording is tracked separately as S4.</t>
+          <t>the widget calls an endpoint that is not present on the deployed build. Either restore centre_head.api.target.main_dashboard.main_target or remove the card that calls it. Either way the frontend should render an explicit empty state rather than the literal string shown today; the broken wording is tracked separately as S4.</t>
         </is>
       </c>
       <c r="M19" s="7" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Client-side auth guard is hardcoded to `true` (disabled)</t>
+          <t>Client-side auth guard is hardcoded to true (disabled)</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>`const isAuthenticated = true;` — the route guard never reads auth state. The redirect-to-login branch is dead code. `URLs.Login` isn't even defined in `routes.js` (would ReferenceError if that branch ever ran).</t>
+          <t>const isAuthenticated = true; — the route guard never reads auth state. The redirect-to-login branch is dead code. URLs.Login isn't even defined in routes.js (would ReferenceError if that branch ever ran).</t>
         </is>
       </c>
       <c r="K20" s="7" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>See register</t>
+          <t>See register.</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>login stores Frappe `api_key`/`api_secret` in `localStorage`; every request sends `Authorization: token &lt;key&gt;:&lt;secret&gt;`.</t>
+          <t>login stores Frappe api_key/api_secret in localStorage; every request sends Authorization: token &lt;key&gt;:&lt;secret&gt;.</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>move the session to a short-lived, `httpOnly`, `Secure`, `SameSite` cookie so it cannot be read from JavaScript, and shorten its lifetime. A token in `localStorage` is readable by any script on the origin — and the persona applications share a single origin, so an XSS in any one of them yields a credential valid for the others.</t>
+          <t>move the session to a short-lived, httpOnly, Secure, SameSite cookie so it cannot be read from JavaScript, and shorten its lifetime. A token in localStorage is readable by any script on the origin — and the persona applications share a single origin, so an XSS in any one of them yields a credential valid for the others.</t>
         </is>
       </c>
       <c r="M21" s="7" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>the full suite executed **three consecutive times**. Each route below rendered nothing in **every** execution, so environmental flake is excluded — routes failing in only some executions are classified separately and are not listed here. Body renders 0 characters.</t>
+          <t>the full suite executed three consecutive times. Each route below rendered nothing in every execution, so environmental flake is excluded — routes failing in only some executions are classified separately and are not listed here. Body renders 0 characters.</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>two independent apps failing on the same two route names points at a shared component (`persona-common-components`) or a shared route-state contract, not at two coincidental per-app bugs. One fix likely clears four failures.</t>
+          <t>two independent apps failing on the same two route names points at a shared component (persona-common-components) or a shared route-state contract, not at two coincidental per-app bugs. One fix likely clears four failures.</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>Verified on the isolated instance (2026-09-20): `youth_skilling.api.curriculum.curriculum_list` returns **HTTP 500** with `TypeError: curriculum_list() missing 1 required positional argument: 'skilling_batch_id'`, and the response carries a traceback. This is therefore an instance of the missing-argument crash pattern rather than a separate defect: give the parameter a default, validate presence explicitly and return **400** naming the missing field. Note the sibling `batch_management.api.curriculum.list` answers **417** to the same shape of call. The two disagree on how a bad request should be rejected.</t>
+          <t>Verified on the isolated instance (2026-09-20): youth_skilling.api.curriculum.curriculum_list returns HTTP 500 with TypeError: curriculum_list() missing 1 required positional argument: 'skilling_batch_id', and the response carries a traceback. This is therefore an instance of the missing-argument crash pattern rather than a separate defect: give the parameter a default, validate presence explicitly and return 400 naming the missing field. Note the sibling batch_management.api.curriculum.list answers 417 to the same shape of call. The two disagree on how a bad request should be rejected.</t>
         </is>
       </c>
       <c r="M24" s="7" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>size the worker pool for the expected concurrency, and return **503** with a retry hint when saturated rather than 500 with a traceback. A 500 tells a client its request was wrong; a 503 tells it to retry, which is the truthful answer under load.</t>
+          <t>size the worker pool for the expected concurrency, and return 503 with a retry hint when saturated rather than 500 with a traceback. A 500 tells a client its request was wrong; a 503 tells it to retry, which is the truthful answer under load.</t>
         </is>
       </c>
       <c r="M25" s="7" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>- **The distribution matters as much as the count.** Four rules fire on **every route scanned, in every persona**. This is not 23 pages each carrying its own mistakes. It is one shared layout and navigation component, repeated across all of them. The 181 orphaned `&lt;li&gt;` elements and the unlabelled icon images match the sidebar navigation observed during route mapping. Impact:** a screen-reader user cannot identify navigation items (no alt text), cannot operate icon-only buttons (no accessible name), and meets a malformed list structure on every page. In practice the platform is not usable with</t>
+          <t>The distribution matters as much as the count. Four rules fire on every route scanned, in every persona. This is not 23 pages each carrying its own mistakes. It is one shared layout and navigation component, repeated across all of them. The 181 orphaned &lt;li&gt; elements and the unlabelled icon images match the sidebar navigation observed during route mapping. Impact: a screen-reader user cannot identify navigation items (no alt text), cannot operate icon-only buttons (no accessible name), and meets a malformed list structure on every page.</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>correct the sidebar list markup (`&lt;li&gt;` inside `&lt;ul&gt;`), add `alt` to nav icons, give icon-only buttons an `aria-label`, and remove ARIA attributes not permitted on their roles — all in the shared navigation component.</t>
+          <t>correct the sidebar list markup (&lt;li&gt; inside &lt;ul&gt;), add alt to nav icons, give icon-only buttons an aria-label, and remove ARIA attributes not permitted on their roles — all in the shared navigation component.</t>
         </is>
       </c>
       <c r="M26" s="7" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>- **Method:** the identical 235-route sweep executed twice, differing only in the number of simultaneous sessions. Same routes, same assertions, same build, minutes apart. - **Note on the two instability figures in this register:** this table reports a controlled comparison of two single executions (3.4% at three sessions, 6.8% at five). The **3.0%** quoted elsewhere is the rate across three consecutive executions at three sessions, which is the more reliable figure and the one used in the client documents. Both describe the platform; they differ in sample size.</t>
+          <t>Method: the identical 235-route sweep executed twice, differing only in the number of simultaneous sessions. Same routes, same assertions, same build, minutes apart. - Note on the two instability figures in this register: this table reports a controlled comparison of two single executions (3.4% at three sessions, 6.8% at five). The 3.0% quoted elsewhere is the rate across three consecutive executions at three sessions, which is the more reliable figure and the one used in the client documents. Both describe the platform; they differ in sample size.</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -3372,7 +3372,7 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>`frappe.utils.change_log.get_versions`, which enumerates the applications **installed on the site**, reports **twelve**: | Source | Applications | Obtainable | |---|---|---| | Framework | `frappe` 15.113.2 · `erpnext` 15.114.0 · `insights` 3.12.5 | Yes — open source | | WeConnect | the eight supplied backends | Yes | | **Vendor** | **`fintoo_analytics_bridge`** | **No** | - **`fintoo_analytics_bridge` exists in no repository in the foundation's GitHub organisation.** The organisation holds eighteen repositories; none corresponds to it. It appears to belong to the development vendor.</t>
+          <t>frappe.utils.change_log.get_versions, which enumerates the applications installed on the site, reports twelve:; Source; Applications; Obtainable; Framework; frappe 15.113.2 · erpnext 15.114.0 · insights 3.12.5; Yes — open source; WeConnect; the eight supplied backends; Yes; Vendor; fintoo_analytics_bridge; No fintoo_analytics_bridge exists in no repository in the foundation's GitHub organisation. The organisation holds eighteen repositories; none corresponds to it. It appears to belong to the development vendor.</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
@@ -3382,7 +3382,7 @@
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
-          <t>(1) establish who owns `fintoo_analytics_bridge` and obtain either the source or a written escrow undertaking. The platform cannot be rebuilt or fully audited without it; (2) declare `required_apps` in each app's `hooks.py` so the deployable set is recorded in code; (3) remove the orphaned `Module Def` records for apps that are not installed (`hrms`, `mannlowe_support`, `materialized_view_builder`), so the installed-application list stops disagreeing with itself.</t>
+          <t>(1) establish who owns fintoo_analytics_bridge and obtain either the source or a written escrow undertaking. The platform cannot be rebuilt or fully audited without it; (2) declare required_apps in each app's hooks.py so the deployable set is recorded in code; (3) remove the orphaned Module Def records for apps that are not installed (hrms, mannlowe_support, materialized_view_builder), so the installed-application list stops disagreeing with itself.</t>
         </is>
       </c>
       <c r="M28" s="7" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>of 297 doctype definitions across the eight applications, **182 carry permission rules and every one of them grants a single role: `System Manager`.** The remaining 115 carry no permission rules at all. **Not one doctype grants any WeConnect role.** - No application defines a `Role` or `Role Profile` record. The declared `fixtures` export only `Custom Field` and `Property Setter`. - Yet the code refers to these roles 227 times — `"Skilling Partner"` alone appears 174 times.</t>
+          <t>of 297 doctype definitions across the eight applications, 182 carry permission rules and every one of them grants a single role: System Manager. The remaining 115 carry no permission rules at all. Not one doctype grants any WeConnect role. - No application defines a Role or Role Profile record. The declared fixtures export only Custom Field and Property Setter. - Yet the code refers to these roles 227 times — "Skilling Partner" alone appears 174 times.</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>- **A pattern, now seen three times.** Standing up the platform from its repositories produces a system that **cannot perform its core flows** until configuration that lives only in the production database is recreated by hand. Concretely, on a clean install: - **Demonstrated, not asserted.** `create_pre_enquiry` — a core Outreach Coordinator flow — returned HTTP 400 "Naming Series mandatory" on a clean install, because `create_youth` does not set a series and none is configured by default. Setting the series made the flow succeed. The stage and status failures were identical.</t>
+          <t>A pattern, now seen three times. Standing up the platform from its repositories produces a system that cannot perform its core flows until configuration that lives only in the production database is recreated by hand. Concretely, on a clean install: - Demonstrated, not asserted. create_pre_enquiry — a core Outreach Coordinator flow — returned HTTP 400 "Naming Series mandatory" on a clean install, because create_youth does not set a series and none is configured by default. Setting the series made the flow succeed. The stage and status failures were identical.</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>ship this configuration as **fixtures** (Frappe's mechanism for exactly this) or as an **install/after_migrate patch**, so a fresh install is a working install. Some patches exist (placement status master data). The pattern should be extended to the naming series, stages, statuses, roles and role profiles the core flows require.</t>
+          <t>ship this configuration as fixtures (Frappe's mechanism for exactly this) or as an install/after_migrate patch, so a fresh install is a working install. Some patches exist (placement status master data). The pattern should be extended to the naming series, stages, statuses, roles and role profiles the core flows require.</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>across the skilling application alone, endpoint logic branches on membership in named roles — `"Skilling Partner" in user_roles` (7×), `"Skilling Manager" in user_roles` (5×), `"Center Head" in roles`, `"System Manager"` and others. But on an instance built from the repositories, **the persona roles do not exist**: `frappe.db.exists("Role", "Skilling Partner")` is false, and no Role, Role Profile or role assignment for any persona is shipped in any app.</t>
+          <t>across the skilling application alone, endpoint logic branches on membership in named roles — "Skilling Partner" in user_roles (7×), "Skilling Manager" in user_roles (5×), "Center Head" in roles, "System Manager" and others. But on an instance built from the repositories, the persona roles do not exist: frappe.db.exists("Role", "Skilling Partner") is false, and no Role, Role Profile or role assignment for any persona is shipped in any app.</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>`facilitator_and_counsellor.api.counselling.actions.mark_as_dropoff` The discrepancy.** Called through the HTTP API as the owning persona, both return **403 PermissionError** (a raw traceback, not the endpoint's own graceful "insufficient permission" message). But every operation the endpoint performs — `has_permission("write")`, the field update, `doc.save()` — **succeeds when run directly as the same user** with `frappe.set_user`. For `skilling_issue.update_issue` the endpoint body is only get_doc, a graceful has_permission check, and save; none of those fails in isolation, yet the API call</t>
+          <t>facilitator_and_counsellor.api.counselling.actions.mark_as_dropoff The discrepancy. Called through the HTTP API as the owning persona, both return 403 PermissionError (a raw traceback, not the endpoint's own graceful "insufficient permission" message). But every operation the endpoint performs — has_permission("write"), the field update, doc.save() — succeeds when run directly as the same user with frappe.set_user.</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>root-cause the rejection in the request-handling layer. Ruled out during investigation: payload format, HTTP verb, roles, centre scope and hooks — and the functions run correctly when invoked directly through `bench`, so the defect is not in the handler body. Until it is located, `update_issue` and `mark_as_dropoff` are unreachable over HTTP for every caller, which makes them both untestable and unusable by the frontends.</t>
+          <t>root-cause the rejection in the request-handling layer. Ruled out during investigation: payload format, HTTP verb, roles, centre scope and hooks — and the functions run correctly when invoked directly through bench, so the defect is not in the handler body. Until it is located, update_issue and mark_as_dropoff are unreachable over HTTP for every caller, which makes them both untestable and unusable by the frontends.</t>
         </is>
       </c>
       <c r="M32" s="7" t="inlineStr">
@@ -3808,7 +3808,7 @@
       <c r="H33" s="7" t="inlineStr">
         <is>
           <t>Inspection, not a runtime reproduction.
-1. Open `youth_skilling/.../doctype/skilling_batch_attendance/skilling_batch_attendance.py:190`, and the same pair of values in `skilling_batch.py:292` and `api/batch_management.py:5418`..
+1. Open youth_skilling/.../doctype/skilling_batch_attendance/skilling_batch_attendance.py:190, and the same pair of values in skilling_batch.py:292 and api/batch_management.py:5418.
 2. Confirm what the Actual Result column describes is present (or absent).
 3. Full reasoning is in findings/findings-log.md under WC-103.</t>
         </is>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>creating any `Skilling Batch Attendance` fails with `Could not find Status: Skilling Not Enrolled`. (The message uses the field's *label*, "Status", not the doctype name `Youth Status` — which makes it actively misleading when diagnosing.) Creating the two missing `Youth Status` records by hand makes attendance work immediately: `mark_attendance` then succeeded and ground truth confirms the row (`Skilling Attendance Table`: `2026-08-05 / Present`).</t>
+          <t>creating any Skilling Batch Attendance fails with Could not find Status: Skilling Not Enrolled. (The message uses the field's *label*, "Status", not the doctype name Youth Status — which makes it actively misleading when diagnosing.) Creating the two missing Youth Status records by hand makes attendance work immediately: mark_attendance then succeeded and ground truth confirms the row (Skilling Attendance Table: 2026-08-05 / Present).</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>ship the `Youth Status` master as app fixtures, including every value the code writes. A test that asserts each status literal in the codebase exists in the master would have caught this.</t>
+          <t>ship the Youth Status master as app fixtures, including every value the code writes. A test that asserts each status literal in the codebase exists in the master would have caught this.</t>
         </is>
       </c>
       <c r="M33" s="7" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>The environment→API mapping is shifted by one in every repository, and no configuration targets a production API</t>
+          <t>The environment -&gt; API mapping is shifted by one in every repository, and no configuration targets a production API</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>This supersedes and sharpens the earlier "UAT frontend calls the DEV backend API" finding, which recorded one symptom. The defect is uniform and it is committed. - **Evidence. Every frontend repository plus the shared component library (9 of 9):</t>
+          <t>This supersedes and sharpens the earlier "UAT frontend calls the DEV backend API" finding, which recorded one symptom. The defect is uniform and it is committed. - Evidence. Every frontend repository plus the shared component library (9 of 9):</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
-          <t>1. Correct the mapping so each environment's config names its own API, and add the missing production configuration. 2. Stop committing `.env*` files; supply them at build time. (Recorded separately as hygiene — contents are now inspected and contain **no credentials**, only URLs, so that finding stays S3.) 3. Retire or rename `lcfuat.ash.frappe.cloud` so one name denotes one environment. 4. Confirm which frontends are deployed from which config today.</t>
+          <t>1. Correct the mapping so each environment's config names its own API, and add the missing production configuration. 2. Stop committing .env* files; supply them at build time. (Recorded separately as hygiene — contents are now inspected and contain no credentials, only URLs, so that finding stays S3.) 3. Retire or rename lcfuat.ash.frappe.cloud so one name denotes one environment. 4. Confirm which frontends are deployed from which config today.</t>
         </is>
       </c>
       <c r="M34" s="7" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>If any such account exists in production, that user cannot use the platform at all — login succeeds and then sends them nowhere. If no such account exists, the backend carries a fully-wired persona with no way to reach it, and the routing table advertises a destination that was never built. Either way the persona inventory the platform implements and the one it ships do not agree. - **`Trainer` is a second gap, of a different kind.** It is a distinct role profile routed to the Skilling Partner application, and the backend treats it specially — `get_user_permitted_centres()` scopes Trainers by the partners that list them, because a Trainer has no `partner_email_id` of its own. **This engagement tested `sp` but never a Trainer**, so that scoping path is unexercised.</t>
+          <t>If any such account exists in production, that user cannot use the platform at all — login succeeds and then sends them nowhere. If no such account exists, the backend carries a fully-wired persona with no way to reach it, and the routing table advertises a destination that was never built. Either way the persona inventory the platform implements and the one it ships do not agree. - Trainer is a second gap, of a different kind. It is a distinct role profile routed to the Skilling Partner application, and the backend treats it specially — get_user_permitted_centres() scopes Trainers by the partners that list them, because a Trainer has no partner_email_id of its own. This engagement tested sp but never a Trainer, so that scoping path is unexercised.</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>1. Decide whether `Placement Youth Coordinator` is a live persona. If it is, the `/pyc/` application is missing and must be built; if it is not, remove it from the routing table, the helper mappings and the approval patches so the code stops advertising it. 2. Make the routing table fail loudly. An unmapped or unbuilt destination should show an error, not redirect a user into a void. 3. Confirm whether any production account holds the `Placement Youth Coordinator` or `Trainer` role profile; both change the tested surface. - **[DECISION for the client]** Is `Placement Youth Coordinator` in scope for QA, and does a `/pyc/` application exist anywhere outside the repositories we were given?</t>
+          <t>1. Decide whether Placement Youth Coordinator is a live persona. If it is, the /pyc/ application is missing and must be built; if it is not, remove it from the routing table, the helper mappings and the approval patches so the code stops advertising it. 2. Make the routing table fail loudly. An unmapped or unbuilt destination should show an error, not redirect a user into a void. 3. Confirm whether any production account holds the Placement Youth Coordinator or Trainer role profile; both change the tested surface. - [DECISION for the client] Is Placement Youth Coordinator in scope for QA, and does a /pyc/ application exist anywhere outside the repositories we were given?</t>
         </is>
       </c>
       <c r="M35" s="7" t="inlineStr">
@@ -4085,7 +4085,7 @@
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>Found by rebuilding the environment from nothing and driving the suite against it. It is the same class as the `Youth Status` defect, and the two together show the pattern is not a one-off. - **The mechanism.** `Approval.validate_approval_category()` (`centre_head/.../doctype/approval/approval.py:103-111`) rejects any approval whose category does not exist with a matching `ref_doc`:</t>
+          <t>Found by rebuilding the environment from nothing and driving the suite against it. It is the same class as the Youth Status defect, and the two together show the pattern is not a one-off. - The mechanism. Approval.validate_approval_category() (centre_head/.../doctype/approval/approval.py:103-111) rejects any approval whose category does not exist with a matching ref_doc:</t>
         </is>
       </c>
       <c r="K36" s="7" t="inlineStr">
@@ -4095,7 +4095,7 @@
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
-          <t>ship the `Approval Category` records as app fixtures, one per literal the code references, each with the correct `ref_doc`. Then replace the string literals with module-level constants so a typo is a failure at import rather than a runtime `throw`, and reconcile the `Another`/`another` pair. A test that asserts every literal resolves to an existing category would keep the two in step. --- # Security coverage gap review against OWASP API Security Top 10 (2026-09-22)</t>
+          <t>ship the Approval Category records as app fixtures, one per literal the code references, each with the correct ref_doc. Then replace the string literals with module-level constants so a typo is a failure at import rather than a runtime throw, and reconcile the Another/another pair. A test that asserts every literal resolves to an existing category would keep the two in step. --- # Security coverage gap review against OWASP API Security Top 10 (2026-09-22)</t>
         </is>
       </c>
       <c r="M36" s="7" t="inlineStr">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>`HEAD https://uat.lighthouseconnect.org/` returns, in full: `Server: nginx/1.24.0 (Ubuntu)`, `Date`, `Content-Type`, `Content-Length`, `Connection`, `Last-Modified`, `ETag`, `Accept-Ranges`. **None of the following is present:** | Header | Absent | What it would prevent | |---|---|---| | `Content-Security-Policy` | yes | Cross-site scripting, and exfiltration of anything readable from the page | | `Strict-Transport-Security` | yes | Protocol downgrade, cookie/token interception on first request | | `X-Frame-Options` / `frame-ancestors` | yes | Clickjacking | | `X-Content-Type-Options` | yes | MIME-type confusion | | `Referrer-Policy` | yes | Leaking authenticated URLs to third parties | | `Permissions-Policy` | yes | Unwanted access to camera, microphone, geolocation |</t>
+          <t>HEAD https://uat.lighthouseconnect.org/ returns, in full: Server: nginx/1.24.0 (Ubuntu), Date, Content-Type, Content-Length, Connection, Last-Modified, ETag, Accept-Ranges. None of the following is present:; Header; Absent; What it would prevent; Content-Security-Policy; yes; Cross-site scripting, and exfiltration of anything readable from the page; Strict-Transport-Security; yes; Protocol downgrade, cookie/token interception on first request; X-Frame-Options / frame-ancestors; yes; Clickjacking; X-Content-Type-Options; yes; MIME-type confusion; Referrer-Policy; yes; Leaking authenticated URLs to third parties; Permissions-Policy; yes; Unwanted access to camera, microphone, geolocation.</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
@@ -4188,7 +4188,7 @@
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>add the headers at the nginx layer serving the frontend. A reasonable starting set is `Strict-Transport-Security` with a long max-age, `X-Content-Type-Options: nosniff`, `Referrer-Policy: strict-origin-when-cross-origin`, `X-Frame-Options: DENY` (or a CSP `frame-ancestors` directive), and a `Content-Security-Policy` developed in report-only mode first so it can be tuned without breaking the applications. Moving the session off `localStorage` and onto the `httpOnly` cookie the API already issues would remove the underlying exposure.</t>
+          <t>add the headers at the nginx layer serving the frontend. A reasonable starting set is Strict-Transport-Security with a long max-age, X-Content-Type-Options: nosniff, Referrer-Policy: strict-origin-when-cross-origin, X-Frame-Options: DENY (or a CSP frame-ancestors directive), and a Content-Security-Policy developed in report-only mode first so it can be tuned without breaking the applications. Moving the session off localStorage and onto the httpOnly cookie the API already issues would remove the underlying exposure.</t>
         </is>
       </c>
       <c r="M37" s="7" t="inlineStr">
@@ -4271,7 +4271,7 @@
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>Forty consecutive authenticated requests to `youth_skilling.api.utils.get_training_center_list` returned **HTTP 200 every time**. No `429`, no `Retry-After`, no throttling of any kind.</t>
+          <t>Forty consecutive authenticated requests to youth_skilling.api.utils.get_training_center_list returned HTTP 200 every time. No 429, no Retry-After, no throttling of any kind.</t>
         </is>
       </c>
       <c r="K38" s="7" t="inlineStr">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
-          <t>apply per-account and per-IP rate limits at the API gateway or in Frappe's own rate-limiting configuration, sized against the concurrency the backend can actually sustain rather than against a theoretical ceiling. Paginate `get_youth_list`. The concurrency defect should be addressed as well, but rate limiting is the control that bounds the damage while it is outstanding.</t>
+          <t>apply per-account and per-IP rate limits at the API gateway or in Frappe's own rate-limiting configuration, sized against the concurrency the backend can actually sustain rather than against a theoretical ceiling. Paginate get_youth_list. The concurrency defect should be addressed as well, but rate limiting is the control that bounds the damage while it is outstanding.</t>
         </is>
       </c>
       <c r="M38" s="7" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>`add_interest` writes any field the caller sends, and saves with permissions switched off</t>
+          <t>add_interest writes any field the caller sends, and saves with permissions switched off</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
@@ -4348,7 +4348,7 @@
       <c r="H39" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as Facilitator and Counsellor.
-2. Call `batch_management/batch_management/api/fc/youth_interest.py:198` `add_interest`. with the fields it documents PLUS one it never mentions.
+2. Call batch_management/batch_management/api/fc/youth_interest.py:198 add_interest with the fields it documents PLUS one it never mentions.
 3. Read the record back from the database and check whether the undeclared field was written.</t>
         </is>
       </c>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>REQD_FIELDS = ("interested_course", "interested_job_role", ...) for i in REQD_FIELDS: if i not in data: ...return # checks these fields are PRESENT ... youth = frappe.get_doc("Youth", youth) youth.update(data) # writes EVERY key the caller sent youth.save(ignore_permissions=True) # no framework permission check `REQD_FIELDS` is a presence check. Nothing rejects keys that are not in it, so `youth.update(data)` applies the caller's whole dictionary to the Youth record.</t>
+          <t>REQD_FIELDS = ("interested_course", "interested_job_role", ...) for i in REQD_FIELDS: if i not in data: ...return # checks these fields are PRESENT ... youth = frappe.get_doc("Youth", youth) youth.update(data) # writes EVERY key the caller sent youth.save(ignore_permissions=True) # no framework permission check REQD_FIELDS is a presence check. Nothing rejects keys that are not in it, so youth.update(data) applies the caller's whole dictionary to the Youth record.</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>Reject unknown keys before the write, the way `youth_skilling/api/skilling_issue.py` `update_issue` already does in this same codebase: for field in data: if field not in EDITABLE_FIELDS: ...reject Then remove `ignore_permissions=True` so the framework check applies, or state in the code why it has to be bypassed.</t>
+          <t>Reject unknown keys before the write, the way youth_skilling/api/skilling_issue.py update_issue already does in this same codebase: for field in data: if field not in EDITABLE_FIELDS: ...reject Then remove ignore_permissions=True so the framework check applies, or state in the code why it has to be bypassed.</t>
         </is>
       </c>
       <c r="M39" s="7" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>Found by adding boundary-value analysis, which the engagement had not previously covered. The earlier validation probe tested wrong *classes* of input — a string where a number belongs, a missing field. It never tested values of the right type that are impossible in context. Why this can be reported before the characterisation baseline is signed.** These are not cases where correct behaviour is a matter of opinion. A negative age, a birth date in the future, a minimum capacity above the maximum, and a negative course cost are wrong on their own terms. No baseline is needed to say so.</t>
+          <t>Found by adding boundary-value analysis, which the engagement had not previously covered. The earlier validation probe tested wrong *classes* of input — a string where a number belongs, a missing field. It never tested values of the right type that are impossible in context. Why this can be reported before the characterisation baseline is signed. These are not cases where correct behaviour is a matter of opinion. A negative age, a birth date in the future, a minimum capacity above the maximum, and a negative course cost are wrong on their own terms. No baseline is needed to say so.</t>
         </is>
       </c>
       <c r="K40" s="7" t="inlineStr">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>Put the constraint on the doctype, not in each endpoint, so every write path inherits it: a `validate` method rejecting negative or absurd ages, birth dates outside a plausible range, capacity inversions, and negative or out-of-range money and percentage values. Frappe supports this directly, and `non_negative` is available on numeric fields for the simplest of them.</t>
+          <t>Put the constraint on the doctype, not in each endpoint, so every write path inherits it: a validate method rejecting negative or absurd ages, birth dates outside a plausible range, capacity inversions, and negative or out-of-range money and percentage values. Frappe supports this directly, and non_negative is available on numeric fields for the simplest of them.</t>
         </is>
       </c>
       <c r="M40" s="7" t="inlineStr">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>Found by adding systematic state-transition testing, which the engagement had not previously covered. The earlier lifecycle and state-boundary probes tested individual journeys; neither enumerated the full transition matrix. Why this can be reported before the characterisation baseline is signed.** We are not asserting which transitions the foundation intends to allow. We are reporting that the platform permits all of them, which means no intended model is being enforced anywhere. That is a structural fact about the system, not a judgement about correct behaviour.</t>
+          <t>Found by adding systematic state-transition testing, which the engagement had not previously covered. The earlier lifecycle and state-boundary probes tested individual journeys; neither enumerated the full transition matrix. Why this can be reported before the characterisation baseline is signed. We are not asserting which transitions the foundation intends to allow. We are reporting that the platform permits all of them, which means no intended model is being enforced anywhere. That is a structural fact about the system, not a judgement about correct behaviour.</t>
         </is>
       </c>
       <c r="K41" s="7" t="inlineStr">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>Define the permitted transitions once, on the doctype, so every write path inherits them. Frappe ships a Workflow facility for exactly this, and it also provides the transition history and approval steps that the invoice states in particular need. Where a full workflow is too heavy, a `validate` method comparing the new status against the previous value is enough to refuse the impossible moves.</t>
+          <t>Define the permitted transitions once, on the doctype, so every write path inherits them. Frappe ships a Workflow facility for exactly this, and it also provides the transition history and approval steps that the invoice states in particular need. Where a full workflow is too heavy, a validate method comparing the new status against the previous value is enough to refuse the impossible moves.</t>
         </is>
       </c>
       <c r="M41" s="7" t="inlineStr">
@@ -4625,7 +4625,7 @@
       <c r="H42" s="7" t="inlineStr">
         <is>
           <t>Inspection, not a runtime reproduction.
-1. Open weconnect-frontend-fc repo, `dev` branch: `.env`, `.env.uat`, `.env.prod` tracked.
+1. Open weconnect-frontend-fc repo, dev branch: .env, .env.uat, .env.prod tracked.
 2. Confirm what the Actual Result column describes is present (or absent).
 3. Full reasoning is in findings/findings-log.md under WC-004.</t>
         </is>
@@ -4637,7 +4637,7 @@
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>hygiene; `.env.prod` should not be committed. (Contents not inspected.)</t>
+          <t>hygiene; .env.prod should not be committed. (Contents not inspected.)</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>supply environment configuration at build time (CI variables or an untracked `.env.local`), keep only a committed `.env.example`, and add `.env*` to `.gitignore` with the example excepted. This also removes the possibility of a credential being added to one of these files later and inherited by every fork and clone.</t>
+          <t>supply environment configuration at build time (CI variables or an untracked .env.local), keep only a committed .env.example, and add .env* to .gitignore with the example excepted. This also removes the possibility of a credential being added to one of these files later and inherited by every fork and clone.</t>
         </is>
       </c>
       <c r="M42" s="7" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>**3,825 records in a single response — 204 KB, 1.82 s.** The response carries a `count` field but no `total_pages` or `total_data_count`, and accepts no page parameter.</t>
+          <t>3,825 records in a single response — 204 KB, 1.82 s. The response carries a count field but no total_pages or total_data_count, and accepts no page parameter.</t>
         </is>
       </c>
       <c r="K43" s="7" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>`move_youth` creates a batch-transfer approval for any youth with no caller check</t>
+          <t>move_youth creates a batch-transfer approval for any youth with no caller check</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>`move_youth` creates a batch-transfer approval for any youth with no caller check</t>
+          <t>move_youth creates a batch-transfer approval for any youth with no caller check.</t>
         </is>
       </c>
       <c r="K44" s="7" t="inlineStr">
@@ -4827,7 +4827,7 @@
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>check the caller's `permitted_centres` against the youth's centre before creating the approval.</t>
+          <t>check the caller's permitted_centres against the youth's centre before creating the approval.</t>
         </is>
       </c>
       <c r="M44" s="7" t="inlineStr">
@@ -4894,7 +4894,7 @@
       <c r="H45" s="7" t="inlineStr">
         <is>
           <t>1. Create a parent record with at least one dependent record attached.
-2. Call `batch_management/api/pathway_batch/form.py`, `mark_as_deleted(ids, remarks)`. to remove the parent.
+2. Call batch_management/api/pathway_batch/form.py, mark_as_deleted(ids, remarks) to remove the parent.
 3. Check what happened to the dependents.</t>
         </is>
       </c>
@@ -4905,7 +4905,7 @@
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>A batch that youth are actively enrolled in can be marked deleted; their links to it become references to a hidden record. Because it is a soft delete the data is not destroyed, which caps the severity — but the operation offers no guard against removing a batch that is in use, and any list that filters on `is_deleted` will silently drop those youths' batch context.</t>
+          <t>A batch that youth are actively enrolled in can be marked deleted; their links to it become references to a hidden record. Because it is a soft delete the data is not destroyed, which caps the severity — but the operation offers no guard against removing a batch that is in use, and any list that filters on is_deleted will silently drop those youths' batch context.</t>
         </is>
       </c>
       <c r="K45" s="7" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>- **Tested by calling each endpoint twice with an identical payload: - **What this means.** None of these endpoints guards against a repeat. A network retry, a double-click, or a client that re-sends after a timeout will re-run the operation and get a success response each time. The API returns HTTP 200 on the second call, so the caller cannot distinguish a retry from a fresh action.</t>
+          <t>Tested by calling each endpoint twice with an identical payload: - What this means. None of these endpoints guards against a repeat. A network retry, a double-click, or a client that re-sends after a timeout will re-run the operation and get a success response each time. The API returns HTTP 200 on the second call, so the caller cannot distinguish a retry from a fresh action.</t>
         </is>
       </c>
       <c r="K46" s="7" t="inlineStr">
@@ -5039,7 +5039,7 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>`dashboard.get_invoice_count` applies no scoping at all and returns a global financial aggregate</t>
+          <t>dashboard.get_invoice_count applies no scoping at all and returns a global financial aggregate</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>the handler calls `frappe.db.count("Skilling Invoice", {"current_status": ...})` with no centre predicate. `frappe.db.count` does not apply permissions, so no scoping occurs by any route. This one genuinely has no filter, unlike its siblings on the same dashboard.</t>
+          <t>the handler calls frappe.db.count("Skilling Invoice", {"current_status": ...}) with no centre predicate. frappe.db.count does not apply permissions, so no scoping occurs by any route. This one genuinely has no filter, unlike its siblings on the same dashboard.</t>
         </is>
       </c>
       <c r="K47" s="7" t="inlineStr">
@@ -5091,7 +5091,7 @@
       </c>
       <c r="L47" s="7" t="inlineStr">
         <is>
-          <t>filter by the caller's permitted centres, as the sibling cards attempt to, and prefer `frappe.get_list`/`get_all` with an explicit centre predicate over `frappe.db.count`.</t>
+          <t>filter by the caller's permitted centres, as the sibling cards attempt to, and prefer frappe.get_list/get_all with an explicit centre predicate over frappe.db.count.</t>
         </is>
       </c>
       <c r="M47" s="7" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
-          <t>`System Settings` reports `session_expiry = 170:00`, which is **170 hours, a little over seven days**. `force_user_to_reset_password = 0` and `minimum_password_score = 2` on Frappe's 0–4 scale, which zxcvbn describes as "somewhat guessable".</t>
+          <t>System Settings reports session_expiry = 170:00, which is 170 hours, a little over seven days. force_user_to_reset_password = 0 and minimum_password_score = 2 on Frappe's 0–4 scale, which zxcvbn describes as "somewhat guessable".</t>
         </is>
       </c>
       <c r="K48" s="7" t="inlineStr">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="L48" s="7" t="inlineStr">
         <is>
-          <t>shorten the session lifetime to something proportionate to a working day, move the credential to the `httpOnly` cookie the API already issues, and raise the minimum password score. None of these requires application changes; they are settings.</t>
+          <t>shorten the session lifetime to something proportionate to a working day, move the credential to the httpOnly cookie the API already issues, and raise the minimum password score. None of these requires application changes; they are settings.</t>
         </is>
       </c>
       <c r="M48" s="7" t="inlineStr">
@@ -5263,7 +5263,7 @@
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>A preflight to `api-dev.lighthouseconnect.org` carrying `Origin: https://evil.example.com` — a domain with no relationship to the foundation — came back `HTTP/2 200` with `access-control-allow-origin: https://evil.example.com` and `access-control-allow-credentials: true`. An unrelated origin is echoed back verbatim and told that credentialed requests are acceptable. This is the signature of `allow_cors` being set to `"*"`: Frappe does not emit a literal `*`, it reflects whatever origin asked.</t>
+          <t>A preflight to api-dev.lighthouseconnect.org carrying Origin: https://evil.example.com — a domain with no relationship to the foundation — came back HTTP/2 200 with access-control-allow-origin: https://evil.example.com and access-control-allow-credentials: true. An unrelated origin is echoed back verbatim and told that credentialed requests are acceptable. This is the signature of allow_cors being set to "*": Frappe does not emit a literal *, it reflects whatever origin asked.</t>
         </is>
       </c>
       <c r="K49" s="7" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="L49" s="7" t="inlineStr">
         <is>
-          <t>Replace `"*"` with the explicit list of frontend origins that need access. `allow_cors` accepts a list, and `set_cors_headers` already compares the incoming origin against it, so this is a configuration edit with no code change: set it to the UAT and production frontend origins and nothing else. Re-run the probe above afterwards and confirm an unrelated origin gets no `access-control-allow-origin` header back.</t>
+          <t>Replace "*" with the explicit list of frontend origins that need access. allow_cors accepts a list, and set_cors_headers already compares the incoming origin against it, so this is a configuration edit with no code change: set it to the UAT and production frontend origins and nothing else. Re-run the probe above afterwards and confirm an unrelated origin gets no access-control-allow-origin header back.</t>
         </is>
       </c>
       <c r="M49" s="7" t="inlineStr">
@@ -5313,7 +5313,7 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>`update_profile` applies caller data to a User record, and its permission check is dead code</t>
+          <t>update_profile applies caller data to a User record, and its permission check is dead code</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
@@ -5344,7 +5344,7 @@
       <c r="H50" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as an authenticated staff account.
-2. Call `outreach/outreach/apis/profile/form.py:74` `update_profile`. with the fields it documents PLUS one it never mentions.
+2. Call outreach/outreach/apis/profile/form.py:74 update_profile with the fields it documents PLUS one it never mentions.
 3. Read the record back from the database and check whether the undeclared field was written.</t>
         </is>
       </c>
@@ -5355,7 +5355,7 @@
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>`update_profile` applies caller data to a User record, and its permission check is dead code</t>
+          <t>update_profile applies caller data to a User record, and its permission check is dead code.</t>
         </is>
       </c>
       <c r="K50" s="7" t="inlineStr">
@@ -5365,7 +5365,7 @@
       </c>
       <c r="L50" s="7" t="inlineStr">
         <is>
-          <t>Add `return` after the 403. Restrict `data` to the profile fields this screen is meant to edit. Check the permission before applying the data rather than after.</t>
+          <t>Add return after the 403. Restrict data to the profile fields this screen is meant to edit. Check the permission before applying the data rather than after.</t>
         </is>
       </c>
       <c r="M50" s="7" t="inlineStr">
@@ -5443,7 +5443,7 @@
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>"Forgot Password?" href="#" — no destination</t>
+          <t>"Forgot Password?" href="#" — no destination.</t>
         </is>
       </c>
       <c r="K51" s="7" t="inlineStr">
@@ -5453,7 +5453,7 @@
       </c>
       <c r="L51" s="7" t="inlineStr">
         <is>
-          <t>point the anchor at the password-reset route, or remove it until that route exists. The backend already exposes `authentication.api.password.send_otp` / `verify_otp` / `reset_password`, so the flow exists server-side and only the entry point is missing. A user who forgets their password currently has no self-service path at all.</t>
+          <t>point the anchor at the password-reset route, or remove it until that route exists. The backend already exposes authentication.api.password.send_otp / verify_otp / reset_password, so the flow exists server-side and only the entry point is missing. A user who forgets their password currently has no self-service path at all.</t>
         </is>
       </c>
       <c r="M51" s="7" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="L52" s="7" t="inlineStr">
         <is>
-          <t>add `autocomplete="current-password"` to the login password input (and `autocomplete="username"` to the identifier field). One attribute each; it restores password manager support and clears the browser console warning.</t>
+          <t>add autocomplete="current-password" to the login password input (and autocomplete="username" to the identifier field). One attribute each; it restores password manager support and clears the browser console warning.</t>
         </is>
       </c>
       <c r="M52" s="7" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>`authentication.api.auth.login` returns HTTP 200 but `role_profile: ""` for the OC account, while all other personas return a populated profile.</t>
+          <t>authentication.api.auth.login returns HTTP 200 but role_profile: "" for the OC account, while all other personas return a populated profile.</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="L53" s="7" t="inlineStr">
         <is>
-          <t>assign the `Outreach Coordinator` role profile to the account, and make the login endpoint refuse — or at minimum log. An authenticated user with no role profile, rather than returning an empty string that callers must interpret.</t>
+          <t>assign the Outreach Coordinator role profile to the account, and make the login endpoint refuse — or at minimum log. An authenticated user with no role profile, rather than returning an empty string that callers must interpret.</t>
         </is>
       </c>
       <c r="M53" s="7" t="inlineStr">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>SP /approvals data API returns 404</t>
+          <t>SP /approvals data API returns 404.</t>
         </is>
       </c>
       <c r="K54" s="7" t="inlineStr">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="L54" s="7" t="inlineStr">
         <is>
-          <t>the Skilling Partner approvals screen calls an endpoint that is absent on the deployed build. Restore it, or repoint the screen at `youth_skilling.api.approval.approval_list`, which serves the same records and is present. Note that endpoint carries its own defect (its scope resolver returns unrestricted for any `System Manager` holder), so repointing alone is not sufficient.</t>
+          <t>the Skilling Partner approvals screen calls an endpoint that is absent on the deployed build. Restore it, or repoint the screen at youth_skilling.api.approval.approval_list, which serves the same records and is present. Note that endpoint carries its own defect (its scope resolver returns unrestricted for any System Manager holder), so repointing alone is not sufficient.</t>
         </is>
       </c>
       <c r="M54" s="7" t="inlineStr">
@@ -5803,7 +5803,7 @@
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>each persona was offered the 67 endpoints exclusive to other personas. Share refused (401/403): | Caller | Read OK | Refused | Refusal rate | |---|---|---|---| | OC | 48 | 0 | **0%** | | CH | 36 | 3 | 8% | | FC | 45 | 7 | 13% | | SYC | 45 | 9 | 16% | | SM | 33 | 11 | 24% | | SP | 33 | 14 | 29% |</t>
+          <t>each persona was offered the 67 endpoints exclusive to other personas. Share refused (401/403):; Caller; Read OK; Refused; Refusal rate; OC; 48; 0; 0%; CH; 36; 3; 8%; FC; 45; 7; 13%; SYC; 45; 9; 16%; SM; 33; 11; 24%; SP; 33; 14; 29%.</t>
         </is>
       </c>
       <c r="K55" s="7" t="inlineStr">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="L55" s="7" t="inlineStr">
         <is>
-          <t>See register</t>
+          <t>See register.</t>
         </is>
       </c>
       <c r="M55" s="7" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>`color-contrast`, serious, 13 routes, 43 elements.</t>
+          <t>color-contrast, serious, 13 routes, 43 elements.</t>
         </is>
       </c>
       <c r="K56" s="7" t="inlineStr">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="L56" s="7" t="inlineStr">
         <is>
-          <t>the failures are concentrated in shared navigation and shared button styles rather than spread across pages, so correcting the palette tokens in the shared component library (`persona-common-components`) fixes most instances at once. Target WCAG AA — 4.5:1 for body text, 3:1 for large text and UI boundaries — and add an automated contrast check to CI so regressions are caught at build time.</t>
+          <t>the failures are concentrated in shared navigation and shared button styles rather than spread across pages, so correcting the palette tokens in the shared component library (persona-common-components) fixes most instances at once. Target WCAG AA — 4.5:1 for body text, 3:1 for large text and UI boundaries — and add an automated contrast check to CI so regressions are caught at build time.</t>
         </is>
       </c>
       <c r="M56" s="7" t="inlineStr">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>`permitted_courses` is a string for half the accounts and an array for the other half</t>
+          <t>permitted_courses is a string for half the accounts and an array for the other half</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>| Account | `permitted_courses` | |---|---| | FC | `array(3)` | | SP | `array(2)` | | SM | `array(11)` | | **CH** | **`"NA"` (string)** | | **SYC** | **`"NA"` (string)** | | **OC** | **`"NA"` (string)** |</t>
+          <t>Account; permitted_courses; FC; array(3); SP; array(2); SM; array(11); CH; "NA" (string); SYC; "NA" (string); OC; "NA" (string)</t>
         </is>
       </c>
       <c r="K57" s="7" t="inlineStr">
@@ -5989,7 +5989,7 @@
       </c>
       <c r="L57" s="7" t="inlineStr">
         <is>
-          <t>return `[]` rather than the sentinel string `"NA"`. A field's type should not depend on its value. `permitted_centres` is correctly an array for every account and is the reference.</t>
+          <t>return [] rather than the sentinel string "NA". A field's type should not depend on its value. permitted_centres is correctly an array for every account and is the reference.</t>
         </is>
       </c>
       <c r="M57" s="7" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>two consecutive logins for the same account. `api_key` is stable; **`api_secret` is regenerated** on each login, and the first secret immediately returns **401**.</t>
+          <t>two consecutive logins for the same account. api_key is stable; api_secret is regenerated on each login, and the first secret immediately returns 401.</t>
         </is>
       </c>
       <c r="K58" s="7" t="inlineStr">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="L58" s="7" t="inlineStr">
         <is>
-          <t>See register</t>
+          <t>See register.</t>
         </is>
       </c>
       <c r="M58" s="7" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>`weconnect-backend-authentication`, `authentication/api/auth.py:185`: `frappe.db.get_value("Employee", {"user_id": user})`. **No Employee doctype is defined by any of the eight backend applications** — 297 definitions under 293 distinct names were enumerated across all of them, and none is Employee. Accounts carry identifiers of the form `HR-EMP-00471`.</t>
+          <t>weconnect-backend-authentication, authentication/api/auth.py:185: frappe.db.get_value("Employee", {"user_id": user}). No Employee doctype is defined by any of the eight backend applications — 297 definitions under 293 distinct names were enumerated across all of them, and none is Employee. Accounts carry identifiers of the form HR-EMP-00471.</t>
         </is>
       </c>
       <c r="K59" s="7" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="L59" s="7" t="inlineStr">
         <is>
-          <t>declare `required_apps` in `authentication/hooks.py`, and record the deployable set in a README. Both are small; the absence of both is what turns a dependency into a trap.</t>
+          <t>declare required_apps in authentication/hooks.py, and record the deployable set in a README. Both are small; the absence of both is what turns a dependency into a trap.</t>
         </is>
       </c>
       <c r="M59" s="7" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>`Module Def` holds records attributed to three applications that `get_versions` does not list as installed: | Application | Orphaned modules | |---|---| | `hrms` | `HR`, `Payroll` | | `mannlowe_support` | `Mannlowe Support` | | `materialized_view_builder` | `Materialized View Builder` |</t>
+          <t>Module Def holds records attributed to three applications that get_versions does not list as installed:; Application; Orphaned modules; hrms; HR, Payroll; mannlowe_support; Mannlowe Support; materialized_view_builder; Materialized View Builder.</t>
         </is>
       </c>
       <c r="K60" s="7" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="L60" s="7" t="inlineStr">
         <is>
-          <t>remove the orphaned `Module Def` records, or reinstall-and-uninstall cleanly.</t>
+          <t>remove the orphaned Module Def records, or reinstall-and-uninstall cleanly.</t>
         </is>
       </c>
       <c r="M60" s="7" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>parsing all 297 doctype definitions across the eight applications yields only 293 distinct names. Three are declared by **both** `batch_management` and `event_management`: | Doctype | Declared by | Module recorded | |---|---|---| | `Categories` | batch_management / event_management | `Batch Management` / `event_management` | | `Event Category` | batch_management / event_management | `Batch Management` / `event_management` | | `Reason For Visit` | batch_management / event_management | `Batch Management` / `event_management` |</t>
+          <t>parsing all 297 doctype definitions across the eight applications yields only 293 distinct names. Three are declared by both batch_management and event_management:; Doctype; Declared by; Module recorded; Categories; batch_management / event_management; Batch Management / event_management; Event Category; batch_management / event_management; Batch Management / event_management; Reason For Visit; batch_management / event_management; Batch Management / event_management.</t>
         </is>
       </c>
       <c r="K61" s="7" t="inlineStr">
@@ -6426,7 +6426,7 @@
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>the platform scopes a user to centres two different ways. | Mechanism | Source of truth | References in code | |---|---|---| | `permitted_centres` | `User Permission` rows with `allow="Lighthouse Centre"`, resolved at login | 89 | | `Employee.custom_center` | a Link field on the session user's `Employee` record | 58 |</t>
+          <t>the platform scopes a user to centres two different ways.; Mechanism; Source of truth; References in code; permitted_centres; User Permission rows with allow="Lighthouse Centre", resolved at login; 89; Employee.custom_center; a Link field on the session user's Employee record; 58.</t>
         </is>
       </c>
       <c r="K62" s="7" t="inlineStr">
@@ -6436,7 +6436,7 @@
       </c>
       <c r="L62" s="7" t="inlineStr">
         <is>
-          <t>derive one from the other, or have write paths consult `permitted_centres` as read paths do.</t>
+          <t>derive one from the other, or have write paths consult permitted_centres as read paths do.</t>
         </is>
       </c>
       <c r="M62" s="7" t="inlineStr">
@@ -6503,7 +6503,7 @@
       <c r="H63" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as an authenticated staff account.
-2. Call `weconnect-backend-batch-management`, `batch_management/fixtures/custom_field.json` — adds `custom_abbr` ("ABBR") to **`Cost Center`** as `fieldtype: Data`, **`reqd: 1`, with no default**. omitting a required argument, or with an argument of the wrong type.
+2. Call weconnect-backend-batch-management, batch_management/fixtures/custom_field.json — adds custom_abbr ("ABBR") to Cost Center as fieldtype: Data, reqd: 1, with no default omitting a required argument, or with an argument of the wrong type.
 3. Read the HTTP status and the response body.</t>
         </is>
       </c>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>A custom field makes ERPNext's Company creation fail</t>
+          <t>A custom field makes ERPNext's Company creation fail.</t>
         </is>
       </c>
       <c r="K63" s="7" t="inlineStr">
@@ -6524,7 +6524,7 @@
       </c>
       <c r="L63" s="7" t="inlineStr">
         <is>
-          <t>give `custom_abbr` a default, or make it non-mandatory and validate it only where the application actually requires it.</t>
+          <t>give custom_abbr a default, or make it non-mandatory and validate it only where the application actually requires it.</t>
         </is>
       </c>
       <c r="M63" s="7" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>- **Observed directly on the isolated instance**, creating a Task through `outreach.apis.task.task.create_task`: - **A rejected write is indistinguishable from an accepted one by status code.** Both return 200. A caller that checks `response.ok` — which is the normal thing to do, and what most HTTP clients encourage — treats a refused creation as a successful one. The record does not exist; the caller believes it does.</t>
+          <t>Observed directly on the isolated instance, creating a Task through outreach.apis.task.task.create_task: - A rejected write is indistinguishable from an accepted one by status code. Both return 200. A caller that checks response.ok — which is the normal thing to do, and what most HTTP clients encourage — treats a refused creation as a successful one. The record does not exist; the caller believes it does.</t>
         </is>
       </c>
       <c r="K64" s="7" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>`update_task` returns a 500 and a traceback when any field is omitted</t>
+          <t>update_task returns a 500 and a traceback when any field is omitted</t>
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr">
@@ -6683,7 +6683,7 @@
       <c r="H65" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as an authenticated staff account.
-2. Call `outreach/apis/task/task.py`, `update_task`. omitting a required argument, or with an argument of the wrong type.
+2. Call outreach/apis/task/task.py, update_task omitting a required argument, or with an argument of the wrong type.
 3. Read the HTTP status and the response body.</t>
         </is>
       </c>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>the handler reads five payload keys by **direct subscript** rather than `.get()`: `subject`, `description`, `assign_to`, `priority`, `exp_end_date`. Omitting any one raises `KeyError`, which the framework returns as **HTTP 500 with a Python traceback** — not a validation message.</t>
+          <t>the handler reads five payload keys by direct subscript rather than .get(): subject, description, assign_to, priority, exp_end_date. Omitting any one raises KeyError, which the framework returns as HTTP 500 with a Python traceback — not a validation message.</t>
         </is>
       </c>
       <c r="K65" s="7" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="L65" s="7" t="inlineStr">
         <is>
-          <t>`data.get(key)` throughout, and return a 400 with the missing field named.</t>
+          <t>data.get(key) throughout, and return a 400 with the missing field named.</t>
         </is>
       </c>
       <c r="M65" s="7" t="inlineStr">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>- **A recurring pattern**, now confirmed on several endpoints: a whitelisted method with required positional parameters returns **HTTP 500 with a traceback** — not a clean 400 — when a parameter is absent, because Frappe raises `TypeError: &lt;fn&gt;() missing N required positional arguments` before the function body runs. - **Why it matters.** A caller that omits a field — or the frontend during a partial update — gets a 500 and a stack trace instead of a validation message naming the missing field. It compounds the traceback-disclosure finding (every one leaks framework paths) and makes the API ho</t>
+          <t>A recurring pattern, now confirmed on several endpoints: a whitelisted method with required positional parameters returns HTTP 500 with a traceback — not a clean 400 — when a parameter is absent, because Frappe raises TypeError: &lt;fn&gt;() missing N required positional arguments before the function body runs. - Why it matters. A caller that omits a field — or the frontend during a partial update — gets a 500 and a stack trace instead of a validation message naming the missing field.</t>
         </is>
       </c>
       <c r="K66" s="7" t="inlineStr">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="L66" s="7" t="inlineStr">
         <is>
-          <t>give optional parameters defaults and validate presence explicitly, returning 400 with the missing field named. This is idiomatic Frappe; the endpoints that get it right (e.g. `create_task` with `.get()`) show the pattern.</t>
+          <t>give optional parameters defaults and validate presence explicitly, returning 400 with the missing field named. This is idiomatic Frappe; the endpoints that get it right (e.g. create_task with .get()) show the pattern.</t>
         </is>
       </c>
       <c r="M66" s="7" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Skilling Invoice `validate()` raises a SQL error on a missing column</t>
+          <t>Skilling Invoice validate() raises a SQL error on a missing column</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
@@ -6870,7 +6870,7 @@
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>- The earlier "observed, not root-caused" invoice SQL error is now located and confirmed as real. Creating a Skilling Invoice through the normal path fails in `validate()` (`Unknown column 'skilling_batch' in 'WHERE'`). The invoice created successfully **only when validate was skipped** (`ignore_validate`). So the invoice controller's validate logic contains a query referencing a column that does not exist in the queried table, and it fires on save. Impact:** invoice creation through the ordinary path is affected by this. It did not block the S1 above (the invoice was seeded with validate skip</t>
+          <t>The earlier "observed, not root-caused" invoice SQL error is now located and confirmed as real. Creating a Skilling Invoice through the normal path fails in validate() (Unknown column 'skilling_batch' in 'WHERE'). The invoice created successfully only when validate was skipped (ignore_validate). So the invoice controller's validate logic contains a query referencing a column that does not exist in the queried table, and it fires on save. Impact: invoice creation through the ordinary path is affected by this.</t>
         </is>
       </c>
       <c r="K67" s="7" t="inlineStr">
@@ -6880,7 +6880,7 @@
       </c>
       <c r="L67" s="7" t="inlineStr">
         <is>
-          <t>the `validate()` query references a column that does not exist on the table it queries (`Unknown column 'skilling_batch' in 'WHERE'`). Correct the column name, or the doctype it queries, so invoice creation through the ordinary path succeeds. A test that creates a Skilling Invoice without `ignore_validate` would have caught this. No such test exists today.</t>
+          <t>the validate() query references a column that does not exist on the table it queries (Unknown column 'skilling_batch' in 'WHERE'). Correct the column name, or the doctype it queries, so invoice creation through the ordinary path succeeds. A test that creates a Skilling Invoice without ignore_validate would have caught this. No such test exists today.</t>
         </is>
       </c>
       <c r="M67" s="7" t="inlineStr">
@@ -6916,7 +6916,7 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>`add_remarks` crashes with an unhandled ValueError on an empty sequence</t>
+          <t>add_remarks crashes with an unhandled ValueError on an empty sequence</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
-          <t>calling it for a youth in the `Standby` stage returned HTTP 500 with `ValueError: max() arg is an empty sequence` — the code calls `max()` over a collection (likely the youth's screening or call records) without handling the empty case.</t>
+          <t>calling it for a youth in the Standby stage returned HTTP 500 with ValueError: max() arg is an empty sequence — the code calls max() over a collection (likely the youth's screening or call records) without handling the empty case.</t>
         </is>
       </c>
       <c r="K68" s="7" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="L68" s="7" t="inlineStr">
         <is>
-          <t>guard the aggregation (`max(seq, default=...)` or an emptiness check).</t>
+          <t>guard the aggregation (max(seq, default=...) or an emptiness check).</t>
         </is>
       </c>
       <c r="M68" s="7" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>`mark_attendance` requires a pre-existing attendance record, and says so only generically</t>
+          <t>mark_attendance requires a pre-existing attendance record, and says so only generically</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>enrolling a youth in the batch's `youth` child table (`Pathway Batch Student`) is **not** sufficient. `_apply_attendance` looks up a `Skilling Batch Attendance` record for (`skilling_batch_id`, `youth`) and returns `"Skilling Batch Attendance record not found for this youth."` when absent; the caller sees the top-level `"Failed to mark attendance."`</t>
+          <t>enrolling a youth in the batch's youth child table (Pathway Batch Student) is not sufficient. _apply_attendance looks up a Skilling Batch Attendance record for (skilling_batch_id, youth) and returns "Skilling Batch Attendance record not found for this youth." when absent; the caller sees the top-level "Failed to mark attendance.".</t>
         </is>
       </c>
       <c r="K69" s="7" t="inlineStr">
@@ -7092,7 +7092,7 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>`db_create.py` assigns undefined identifiers as database connection settings</t>
+          <t>db_create.py assigns undefined identifiers as database connection settings</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
@@ -7123,7 +7123,7 @@
       <c r="H70" s="7" t="inlineStr">
         <is>
           <t>Inspection, not a runtime reproduction.
-1. Open `Lighthouse-Communities-Foundation/data-pipeline-dashboard`, `db_create.py:4-8`..
+1. Open Lighthouse-Communities-Foundation/data-pipeline-dashboard, db_create.py:4-8.
 2. Confirm what the Actual Result column describes is present (or absent).
 3. Full reasoning is in findings/findings-log.md under WC-108.</t>
         </is>
@@ -7135,7 +7135,7 @@
       </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>`DB_HOST = yor_host_name`, `DB_NAME = database_name`, `DB_USER = user_name`, `DB_PASSWORD = db_password` — bare identifiers, not strings, so the module raises `NameError` on import. Note the typo `yor_host_name`.</t>
+          <t>DB_HOST = yor_host_name, DB_NAME = database_name, DB_USER = user_name, DB_PASSWORD = db_password — bare identifiers, not strings, so the module raises NameError on import. Note the typo yor_host_name.</t>
         </is>
       </c>
       <c r="K70" s="7" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="L70" s="7" t="inlineStr">
         <is>
-          <t>read these from the environment (`os.environ`), as the Google credentials already are, and remove the placeholders.</t>
+          <t>read these from the environment (os.environ), as the Google credentials already are, and remove the placeholders.</t>
         </is>
       </c>
       <c r="M70" s="7" t="inlineStr">
@@ -7223,7 +7223,7 @@
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>Tested in response to the OWASP coverage gap at API3 (Broken Object Property Level Authorization), which had not been examined. The result is mixed rather than clean. - **Method.** As the owning persona, create a record through the normal endpoint, then attempt to set protected or system-controlled properties through the endpoint's `data` payload, then read the record back from the database to see what actually persisted. Fields attempted: `owner`, `docstatus`, the centre link, and the workflow status.</t>
+          <t>Tested in response to the OWASP coverage gap at API3 (Broken Object Property Level Authorization), which had not been examined. The result is mixed rather than clean. - Method. As the owning persona, create a record through the normal endpoint, then attempt to set protected or system-controlled properties through the endpoint's data payload, then read the record back from the database to see what actually persisted. Fields attempted: owner, docstatus, the centre link, and the workflow status.</t>
         </is>
       </c>
       <c r="K71" s="7" t="inlineStr">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="L71" s="7" t="inlineStr">
         <is>
-          <t>adopt the Pre Enquiry allowlist pattern across every endpoint that accepts a `data` payload, and add a test asserting that a system-controlled property such as `owner` or `docstatus` cannot be set through any of them.</t>
+          <t>adopt the Pre Enquiry allowlist pattern across every endpoint that accepts a data payload, and add a test asserting that a system-controlled property such as owner or docstatus cannot be set through any of them.</t>
         </is>
       </c>
       <c r="M71" s="7" t="inlineStr">
@@ -7322,7 +7322,7 @@
       </c>
       <c r="L72" s="7" t="inlineStr">
         <is>
-          <t>return 429 with a `Retry-After` header rather than 500. Review whether the per-IP tracker is appropriate for a deployment where many legitimate users share an address, and if it is retained, set its threshold well above the per-account one.</t>
+          <t>return 429 with a Retry-After header rather than 500. Review whether the per-IP tracker is appropriate for a deployment where many legitimate users share an address, and if it is retained, set its threshold well above the per-account one.</t>
         </is>
       </c>
       <c r="M72" s="7" t="inlineStr">
@@ -7401,7 +7401,7 @@
       </c>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>login requests `/src/assets/icons/logo_transparent.png` (unbundled source path)</t>
+          <t>login requests /src/assets/icons/logo_transparent.png (unbundled source path)</t>
         </is>
       </c>
       <c r="K73" s="7" t="inlineStr">
@@ -7411,7 +7411,7 @@
       </c>
       <c r="L73" s="7" t="inlineStr">
         <is>
-          <t>import the asset so the bundler fingerprints and rewrites its path, rather than referencing `/src/...` literally. As shipped the path only resolves by accident of how the site is served, and will 404 under any stricter static configuration.</t>
+          <t>import the asset so the bundler fingerprints and rewrites its path, rather than referencing /src/... literally. As shipped the path only resolves by accident of how the site is served, and will 404 under any stricter static configuration.</t>
         </is>
       </c>
       <c r="M73" s="7" t="inlineStr">
@@ -7589,7 +7589,7 @@
       </c>
       <c r="L75" s="7" t="inlineStr">
         <is>
-          <t>opt in to the v7 behaviours now (`v7_startTransition`, `v7_relativeSplatPath`) so the eventual upgrade is a no-op, or pin the router version and record the decision. Console noise is the visible symptom; the real cost is that genuine warnings are lost among it.</t>
+          <t>opt in to the v7 behaviours now (v7_startTransition, v7_relativeSplatPath) so the eventual upgrade is a no-op, or pin the router version and record the decision. Console noise is the visible symptom; the real cost is that genuine warnings are lost among it.</t>
         </is>
       </c>
       <c r="M75" s="7" t="inlineStr">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="J76" s="7" t="inlineStr">
         <is>
-          <t>FC nav links use `/fc/fc/all-batches`, `/fc/fc/counselling`, `/fc/fc/tasks` (double `fc`). Works, but smells like a base-path bug. ---</t>
+          <t>FC nav links use /fc/fc/all-batches, /fc/fc/counselling, /fc/fc/tasks (double fc). Works, but smells like a base-path bug.</t>
         </is>
       </c>
       <c r="K76" s="7" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="L76" s="7" t="inlineStr">
         <is>
-          <t>the navigation links include the base path that the router already applies, producing `/fc/fc/...`. Make the links relative to the router base, or drop the base from the `basename` configuration — one or the other, not both. It works today only because the server tolerates the duplicated segment.</t>
+          <t>the navigation links include the base path that the router already applies, producing /fc/fc/.... Make the links relative to the router base, or drop the base from the basename configuration — one or the other, not both. It works today only because the server tolerates the duplicated segment.</t>
         </is>
       </c>
       <c r="M76" s="7" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Dead anchors (`href="#"`) in navigation</t>
+          <t>Dead anchors (href="#") in navigation</t>
         </is>
       </c>
       <c r="C77" s="12" t="inlineStr">
@@ -7766,7 +7766,7 @@
       </c>
       <c r="L77" s="7" t="inlineStr">
         <is>
-          <t>give each anchor a real destination, or use a `&lt;button&gt;` where the element triggers an action rather than navigation. An `href="#"` is announced to assistive technology as a link that goes nowhere, and it scrolls the page to the top when activated — so this is an accessibility defect as well as a cosmetic one.</t>
+          <t>give each anchor a real destination, or use a &lt;button&gt; where the element triggers an action rather than navigation. An href="#" is announced to assistive technology as a link that goes nowhere, and it scrolls the page to the top when activated — so this is an accessibility defect as well as a cosmetic one.</t>
         </is>
       </c>
       <c r="M77" s="7" t="inlineStr">
@@ -7833,7 +7833,7 @@
       <c r="H78" s="7" t="inlineStr">
         <is>
           <t>Inspection, not a runtime reproduction.
-1. Open `/oc/test-zustand`, defined in the OC application's router and reachable in UAT..
+1. Open /oc/test-zustand, defined in the OC application's router and reachable in UAT.
 2. Confirm what the Actual Result column describes is present (or absent).
 3. Full reasoning is in findings/findings-log.md under WC-041.</t>
         </is>
@@ -7922,7 +7922,7 @@
       <c r="H79" s="7" t="inlineStr">
         <is>
           <t>Inspection, not a runtime reproduction.
-1. Open `weconnect-backend-outreach` - `outreach/outreach/doctype/google_form_settings/google_form_settings.json` - `outreach/outreach/doctype/google_integration_settings/google_integration_settings.json`.
+1. Open weconnect-backend-outreach - outreach/outreach/doctype/google_form_settings/google_form_settings.json - outreach/outreach/doctype/google_integration_settings/google_integration_settings.json.
 2. Confirm what the Actual Result column describes is present (or absent).
 3. Full reasoning is in findings/findings-log.md under WC-063.</t>
         </is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="J79" s="7" t="inlineStr">
         <is>
-          <t>both files declare `"name": "Google Integration Settings"` with identical fields. The modification stamps — `2026-03-05` and `2026-05-26` — show the doctype was renamed and the original folder was never deleted. Only the newer name is referenced in code (`outreach/api.py:176`, `apis/lcf_mastersheet_sync.py:236`); `Google Form Settings` is referenced nowhere.</t>
+          <t>both files declare "name": "Google Integration Settings" with identical fields. The modification stamps — 2026-03-05 and 2026-05-26 — show the doctype was renamed and the original folder was never deleted. Only the newer name is referenced in code (outreach/api.py:176, apis/lcf_mastersheet_sync.py:236); Google Form Settings is referenced nowhere.</t>
         </is>
       </c>
       <c r="K79" s="7" t="inlineStr">
@@ -7944,7 +7944,7 @@
       </c>
       <c r="L79" s="7" t="inlineStr">
         <is>
-          <t>delete the `google_form_settings/` folder.</t>
+          <t>delete the google_form_settings/ folder.</t>
         </is>
       </c>
       <c r="M79" s="7" t="inlineStr">
@@ -8011,7 +8011,7 @@
       <c r="H80" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as an authenticated staff account — any authenticated account is enough.
-2. Call `outreach/apis/registration/files.py` `upload_file`, and the sibling `facilitator_and_counsellor/api/registration_form_B/files.py`. with no special privileges.
+2. Call outreach/apis/registration/files.py upload_file, and the sibling facilitator_and_counsellor/api/registration_form_B/files.py with no special privileges.
 3. Observe that the call is accepted rather than refused, and check whether anything changed.</t>
         </is>
       </c>
@@ -8077,7 +8077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8158,7 +8158,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Project foundation, architecture, scope, methodology. • Phase 1 baseline, findings register, three graphs. • Reachability figures replaced with single-run verified results (219/235, 93.2%; 16 persistent failures; 9 retr • RBAC read-leakage complete (§7a): 318 probes, no cross-persona data leakage, unauthenticated access refused on</t>
+          <t>Project foundation, architecture, scope, methodology • Phase 1 baseline, findings register, three graphs • Reachability figures replaced with single-run verified results (219/235, 93.2%; 16 persistent failures; 9 retries) superseding the earlier stitched 214/235. Shared-component defect cluster added (§7). PM reclassified from "awaiting credentials" to "deferred — under development" (§3, §9). SP notes corrected: approvals renders and is an API-contract defect, not a blank page. BrowserStack capacity constraint added with measured costings (§10.4). Test architecture section added (§5). Phase 1 category status table added (§6). Constraints register added (§9) • RBAC read-leakage complete (§7a): 318 probes, no cross-persona data leakage, unauthenticated access refused on all 23 probes. Two new defects — S2 stack-trace disclosure, S3 inconsistent endpoint authorization … (full detail in the findings register)</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -8188,12 +8188,12 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Project foundation, architecture, scope, methodology. • Phase 1 baseline, findings register, three graphs. • Reachability figures replaced with single-run verified results (219/235, 93.2%; 16 persistent failures; 9 retr • RBAC read-leakage complete (§7a): 318 probes, no cross-persona data leakage, unauthenticated access refused on</t>
+          <t>Project foundation, architecture, scope, methodology • Phase 1 baseline, findings register, three graphs • Reachability figures replaced with single-run verified results (219/235, 93.2%; 16 persistent failures; 9 retries) superseding the earlier stitched 214/235. Shared-component defect cluster added (§7). PM reclassified from "awaiting credentials" to "deferred — under development" (§3, §9). SP notes corrected: approvals renders and is an API-contract defect, not a blank page. BrowserStack capacity constraint added with measured costings (§10.4). Test architecture section added (§5). Phase 1 category status table added (§6). Constraints register added (§9) • RBAC read-leakage complete (§7a): 318 probes, no cross-persona data leakage, unauthenticated access refused on all 23 probes. Two new defects — S2 stack-trace disclosure, S3 inconsistent endpoint authorization … (full detail in the findings register)</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Characterisation document issued for sign-off. Completeness audit of Phase 1 found two gaps in our own work: t • Full-coverage sweep complete: all 235 routes now carry reachability, asset-integrity and accessibility checks  • Stability criterion raised: repeated execution is now used to make each route's *classification* deterministic • Auth-guard regression complete (§7b): defect scoped to FC and CH only, correcting the earlier platform-wide as • Asset/link integrity complete (§7d): 373 asset requests, zero failures; one earlier finding no longer reproduc • Self-verification suite added (§7g): 27 controls proving each check detects the condition it reports and ignor • §7a corrected and a previously reported clean result retracted. • Dynamic-route coverage complete (§7h): 11 of 17 covered, 6 blocked on client-supplied identifiers. Invoice pre • Known-defect registry introduced: the suite can now stay green while open defects remain, so a regression is v</t>
+          <t>Characterisation document issued for sign-off. Completeness audit of Phase 1 found two gaps in our own work: the unified sweep had dropped the uncaught-JavaScript-error assertion carried by the suite it replaced, and the self-verification suite was being collected by the main configuration. Both corrected. Two findings added from the audit: a developer test route in the deployed OC application, and coming-soon placeholders confirming some screens are intentionally incomplete. Findings register 38 -&gt; 40 • Full-coverage sweep complete: all 235 routes now carry reachability, asset-integrity and accessibility checks in a single 22-minute pass, replacing the earlier 13% samples. Root cause of the blank routes established — uncaught null dereferences on React Router navigation state — which corrects the earlier "wholly broken" classification and makes the fix specific … (full detail in the findings register)</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
@@ -8223,12 +8223,12 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Characterisation document issued for sign-off. Completeness audit of Phase 1 found two gaps in our own work: t • Full-coverage sweep complete: all 235 routes now carry reachability, asset-integrity and accessibility checks  • Stability criterion raised: repeated execution is now used to make each route's *classification* deterministic • Auth-guard regression complete (§7b): defect scoped to FC and CH only, correcting the earlier platform-wide as • Asset/link integrity complete (§7d): 373 asset requests, zero failures; one earlier finding no longer reproduc • Self-verification suite added (§7g): 27 controls proving each check detects the condition it reports and ignor • §7a corrected and a previously reported clean result retracted. • Dynamic-route coverage complete (§7h): 11 of 17 covered, 6 blocked on client-supplied identifiers. Invoice pre • Known-defect registry introduced: the suite can now stay green while open defects remain, so a regression is v</t>
+          <t>Characterisation document issued for sign-off. Completeness audit of Phase 1 found two gaps in our own work: the unified sweep had dropped the uncaught-JavaScript-error assertion carried by the suite it replaced, and the self-verification suite was being collected by the main configuration. Both corrected. Two findings added from the audit: a developer test route in the deployed OC application, and coming-soon placeholders confirming some screens are intentionally incomplete. Findings register 38 -&gt; 40 • Full-coverage sweep complete: all 235 routes now carry reachability, asset-integrity and accessibility checks in a single 22-minute pass, replacing the earlier 13% samples. Root cause of the blank routes established — uncaught null dereferences on React Router navigation state — which corrects the earlier "wholly broken" classification and makes the fix specific … (full detail in the findings register)</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Phase 2 opened (§13). Write-safety harness built and verified — self-verification 36 → 46 controls. Write surf • Phase 2 feasibility spike succeeded. • Installed-application count corrected from fifteen to twelve, and the unobtainable set from three applications to one. • Environment drift eliminated and verified. • Phase 2 write testing began. Persona accounts built on the isolated instance with disjoint centre scopes; writ • Phase 2 write testing deepened. **Second S1 confirmed end-to-end:** a persona with no permission for a centre  • Phase 2 breadth extended to **8 objects** (Task, Pre Enquiry, Enquiry Form, Counselling, Approval, Follow Up,  • Phase 2 depth complete. • Phase 2 complete — all nine exit criteria met. • Full re-audit of the register, and a correction to our own scoring.</t>
+          <t>Phase 2 opened (§13). Write-safety harness built and verified — self-verification 36 -&gt; 46 controls. Write surface analysed: 814 endpoint references across six applications, 106 distinct write candidates, 103 confirmed mutating across 21 objects. ~~Feasibility spike established that the platform runs fifteen applications, not eight; three are vendor-owned and absent.~~ *(corrected in 1.25: twelve installed, one vendor application absent.)* A correction made earlier in the day — that the backend was pure Frappe — was itself wrong and has been withdrawn; ERPNext 15.114.0 is installed. §11 next steps rewritten, having still listed completed Phase 1 work • Phase 2 feasibility spike succeeded. • Installed-application count corrected from fifteen to twelve, and the unobtainable set from three applications to one. • Environment drift eliminated and verified. • Phase 2 write testing began … (full detail in the findings register)</t>
         </is>
       </c>
       <c r="E7" s="7" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Phase 2 opened (§13). Write-safety harness built and verified — self-verification 36 → 46 controls. Write surf • Phase 2 feasibility spike succeeded. • Installed-application count corrected from fifteen to twelve, and the unobtainable set from three applications to one. • Environment drift eliminated and verified. • Phase 2 write testing began. Persona accounts built on the isolated instance with disjoint centre scopes; writ • Phase 2 write testing deepened. **Second S1 confirmed end-to-end:** a persona with no permission for a centre  • Phase 2 breadth extended to **8 objects** (Task, Pre Enquiry, Enquiry Form, Counselling, Approval, Follow Up,  • Phase 2 depth complete. • Phase 2 complete — all nine exit criteria met. • Full re-audit of the register, and a correction to our own scoring.</t>
+          <t>Phase 2 opened (§13). Write-safety harness built and verified — self-verification 36 -&gt; 46 controls. Write surface analysed: 814 endpoint references across six applications, 106 distinct write candidates, 103 confirmed mutating across 21 objects. ~~Feasibility spike established that the platform runs fifteen applications, not eight; three are vendor-owned and absent.~~ *(corrected in 1.25: twelve installed, one vendor application absent.)* A correction made earlier in the day — that the backend was pure Frappe — was itself wrong and has been withdrawn; ERPNext 15.114.0 is installed. §11 next steps rewritten, having still listed completed Phase 1 work • Phase 2 feasibility spike succeeded. • Installed-application count corrected from fifteen to twelve, and the unobtainable set from three applications to one. • Environment drift eliminated and verified. • Phase 2 write testing began … (full detail in the findings register)</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -8316,42 +8316,67 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Day 6</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Every client-facing document corrected and re-dated, the client already holding the repository. • Repository found public and made private; mass-assignment analysis corrected; verification extended to every P1; permission model drafted.</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Defect tracker produced in the format the client asked for, and the repository found public a second time.</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Day 6</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Defect tracker produced in the format the client asked for, and the repository found public a second time.</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Defect tracker produced in the format requested. Repository found public a second time and set private again.</t>
         </is>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E11" s="9" t="n">
         <v>119</v>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>Repository visibility changed back to public on 28 Sep; set private again today. Needs a cause.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Add one row per working day. The pale rows are yours to continue.</t>
         </is>
@@ -8963,7 +8988,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>- **Source:** `src/routes.js`. ~56 routes are deep-link only (not surfaced in navigation). Impact on QA:** clicking the UI would have found ~7% of screens. Hidden routes (e.g. `/fc/batch-finish/remarks`, `/fc/job-application-edit`, `/fc/view-form-b`) are prime spots for missing auth/validation. These become the test target list.</t>
+          <t>Source: src/routes.js. ~56 routes are deep-link only (not surfaced in navigation). Impact on QA: clicking the UI would have found ~7% of screens. Hidden routes (e.g. /fc/batch-finish/remarks, /fc/job-application-edit, /fc/view-form-b) are prime spots for missing auth/validation. These become the test target list.</t>
         </is>
       </c>
     </row>
@@ -8985,7 +9010,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Status:** the client confirmed PM is still being built. Excluded from QA scope by agreement rather than blocked on a credential. Testing an in-flight build produces findings that are obsolete before they are read. Re-entry condition:** client declares PM feature-complete → request a login, run the same Phase 1 categories against its 46 routes. Route inventory is already captured in `data/routes/pm.json`, so restarting costs nothing.</t>
+          <t>Status: the client confirmed PM is still being built. Excluded from QA scope by agreement rather than blocked on a credential. Testing an in-flight build produces findings that are obsolete before they are read. Re-entry condition: client declares PM feature-complete -&gt; request a login, run the same Phase 1 categories against its 46 routes. Route inventory is already captured in data/routes/pm.json, so restarting costs nothing.</t>
         </is>
       </c>
     </row>
@@ -9007,7 +9032,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>- Correction to earlier assumption. OC app renders fine at /oc/. Earlier "OC broken" was a test-harness prefix error, now fixed. OC's empty role_profile (F13) does not block the app.</t>
+          <t>Correction to earlier assumption. OC app renders fine at /oc/. Earlier "OC broken" was a test-harness prefix error, now fixed. OC's empty role_profile (F13) does not block the app.</t>
         </is>
       </c>
     </row>
@@ -9029,7 +9054,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>- CH 22/22 pass · SM 40/40 pass · SP 25/27 · SYC 44/50 · FC 43/56 · OC (re-running at /oc/) --- # Phase 1 category 2 — RBAC read-leakage (2026-09-18)</t>
+          <t>CH 22/22 pass · SM 40/40 pass · SP 25/27 · SYC 44/50 · FC 43/56 · OC (re-running at /oc/) --- # Phase 1 category 2 — RBAC read-leakage (2026-09-18)</t>
         </is>
       </c>
     </row>
@@ -9051,7 +9076,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>- Existing defects surfaced by the control baseline; they are excluded from the access verdict because a broken endpoint cannot demonstrate anything about permissions. Overlaps the 500/404 findings already recorded. --- # Phase 1 category 4 — Accessibility baseline (2026-09-18)</t>
+          <t>Existing defects surfaced by the control baseline; they are excluded from the access verdict because a broken endpoint cannot demonstrate anything about permissions. Overlaps the 500/404 findings already recorded. --- # Phase 1 category 4 — Accessibility baseline (2026-09-18)</t>
         </is>
       </c>
     </row>
@@ -9073,7 +9098,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>- axe-core detects roughly **30–40%** of WCAG issues. Everything above is a genuine defect, but a clean axe run would not mean the platform is accessible. Keyboard traversal, focus order, screen-reader semantics and colour-in-context still require a manual pass, which is **not** in the current scope. This is stated so the baseline is not read as full accessibility assurance. Gate policy:** the suite fails on `critical` only; serious/moderate/minor are recorded as a prioritised backlog. A suite that fails on every severity from day one gets ignored, and an ignored suite protects nothing.</t>
+          <t>axe-core detects roughly 30–40% of WCAG issues. Everything above is a genuine defect, but a clean axe run would not mean the platform is accessible. Keyboard traversal, focus order, screen-reader semantics and colour-in-context still require a manual pass, which is not in the current scope. This is stated so the baseline is not read as full accessibility assurance. Gate policy: the suite fails on critical only; serious/moderate/minor are recorded as a prioritised backlog. A suite that fails on every severity from day one gets ignored, and an ignored suite protects nothing.</t>
         </is>
       </c>
     </row>
@@ -9095,7 +9120,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>- **Method:** each of the 16 persistent failures was loaded directly, then reached again by client-side navigation from the working application root (`history.pushState` + `popstate`, which is what a React Router link does). Result:** **14 render nothing by either path.** These are broken screens, not deep-link defects — which simplifies the remediation: there is no router-state subtlety to chase.</t>
+          <t>Method: each of the 16 persistent failures was loaded directly, then reached again by client-side navigation from the working application root (history.pushState + popstate, which is what a React Router link does). Result: 14 render nothing by either path. These are broken screens, not deep-link defects — which simplifies the remediation: there is no router-state subtlety to chase.</t>
         </is>
       </c>
     </row>
@@ -9107,7 +9132,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>`batch_list` flagged but NOT an unambiguous violation</t>
+          <t>batch_list flagged but NOT an unambiguous violation</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -9117,7 +9142,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>- Batch records carry a `training_centers[]` array, and CH and SYC see entries naming centres outside their permitted list. **However, zero batch records were wholly outside scope** — every one included at least one centre the caller is permitted for. A batch spanning several centres legitimately names all of them. Recorded as characterisation, not a defect. Confirming intent is a question for the client.</t>
+          <t>Batch records carry a training_centers[] array, and CH and SYC see entries naming centres outside their permitted list. However, zero batch records were wholly outside scope — every one included at least one centre the caller is permitted for. A batch spanning several centres legitimately names all of them. Recorded as characterisation, not a defect. Confirming intent is a question for the client.</t>
         </is>
       </c>
     </row>
@@ -9129,7 +9154,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>`utils.get_training_center_list` returns the full centre list to every persona</t>
+          <t>utils.get_training_center_list returns the full centre list to every persona</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -9139,7 +9164,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>- The response is a reference list of centre names. A picker, not records. FC sees 5 centres beyond its permitted set, CH sees 8. Not a record disclosure. It does expose the organisation's centre structure to every account, so it is recorded for the client to confirm as intended.</t>
+          <t>The response is a reference list of centre names. A picker, not records. FC sees 5 centres beyond its permitted set, CH sees 8. Not a record disclosure. It does expose the organisation's centre structure to every account, so it is recorded for the client to confirm as intended.</t>
         </is>
       </c>
     </row>
@@ -9151,7 +9176,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Four applications ship `coming-soon` placeholder screens</t>
+          <t>Four applications ship coming-soon placeholder screens</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -9161,7 +9186,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>- **Where:** SP, SYC, SM and OC each define a `coming-soon` route. Why it is recorded:** it establishes that some screens are intentionally incomplete. This bears directly on the sixteen blank routes: a subset may be unbuilt features rather than defects. Resolving which is a client decision, raised as item 10.1 in the characterisation document.</t>
+          <t>Where: SP, SYC, SM and OC each define a coming-soon route. Why it is recorded: it establishes that some screens are intentionally incomplete. This bears directly on the sixteen blank routes: a subset may be unbuilt features rather than defects. Resolving which is a client decision, raised as item 10.1 in the characterisation document.</t>
         </is>
       </c>
     </row>
@@ -9183,7 +9208,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>- **182 of 235 routes** carry violations; **3,593 elements** in total. Four rules fire on **every single affected route (182/182)**: `aria-allowed-attr` (808 elements), `image-alt` (428), `listitem` (1,452), `list` (182). Sampling 30 routes suggested this pattern; full coverage confirms it exactly. These are one shared navigation component repeated across every screen of every application.</t>
+          <t>182 of 235 routes carry violations; 3,593 elements in total. Four rules fire on every single affected route (182/182): aria-allowed-attr (808 elements), image-alt (428), listitem (1,452), list (182). Sampling 30 routes suggested this pattern; full coverage confirms it exactly. These are one shared navigation component repeated across every screen of every application.</t>
         </is>
       </c>
     </row>
@@ -9205,7 +9230,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>- **2,157 asset requests across all 235 routes. Zero failures.** No missing assets, no unbundled source paths. The earlier clean result on a 33-route sample holds across the full inventory.</t>
+          <t>2,157 asset requests across all 235 routes. Zero failures. No missing assets, no unbundled source paths. The earlier clean result on a 33-route sample holds across the full inventory.</t>
         </is>
       </c>
     </row>
@@ -9227,7 +9252,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>- **Method:** the full 235-route sweep executed three consecutive times. A route is judged on how it behaves across all three, not on any single run, because a platform that fails intermittently cannot be characterised by one observation. - **Measured instability: 3.0%** of routes behaved inconsistently across the three executions at three concurrent sessions. That figure describes the platform, not the suite.</t>
+          <t>Method: the full 235-route sweep executed three consecutive times. A route is judged on how it behaves across all three, not on any single run, because a platform that fails intermittently cannot be characterised by one observation. - Measured instability: 3.0% of routes behaved inconsistently across the three executions at three concurrent sessions. That figure describes the platform, not the suite.</t>
         </is>
       </c>
     </row>
@@ -9249,7 +9274,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>- **`/fc/daily-activity`** was added to the known-defect registry on the strength of a single sweep. Across three consecutive executions it rendered every time. It was one flake, recorded as a defect. **Removed. `/all-notifications`** was identified after two cycles as an unrecorded defect. The third cycle showed it rendering; single-session runs confirmed it. **Classified environmental, not a defect.</t>
+          <t>/fc/daily-activity was added to the known-defect registry on the strength of a single sweep. Across three consecutive executions it rendered every time. It was one flake, recorded as a defect. Removed. /all-notifications was identified after two cycles as an unrecorded defect. The third cycle showed it rendering; single-session runs confirmed it. Classified environmental, not a defect.</t>
         </is>
       </c>
     </row>
@@ -9271,7 +9296,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>- Every one of the 14 registered blank routes is blank in all three executions, and every route blank in all three executions is registered. Verified programmatically, not by inspection.</t>
+          <t>Every one of the 14 registered blank routes is blank in all three executions, and every route blank in all three executions is registered. Verified programmatically, not by inspection.</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9318,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>- The two invoice preparation routes were asserted to attempt exactly the registered `prepare_tax_invoice` POST on load. Those assertions **passed in all three cycles**, meaning the write was attempted every time and no *additional* mutating request occurred. The finding is therefore reproducible, and its scope is bounded: one endpoint, two routes, no other writes anywhere in 235 routes × 3 executions.</t>
+          <t>The two invoice preparation routes were asserted to attempt exactly the registered prepare_tax_invoice POST on load. Those assertions passed in all three cycles, meaning the write was attempted every time and no *additional* mutating request occurred. The finding is therefore reproducible, and its scope is bounded: one endpoint, two routes, no other writes anywhere in 235 routes × 3 executions.</t>
         </is>
       </c>
     </row>
@@ -9315,7 +9340,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>- Earlier the claim rested on 23 probes. **All 71 distinct endpoints observed in use were then probed with no credential: every one returned 403, none served data. The claim "no observed endpoint serves data to an unauthenticated caller" is now complete across the observed endpoint set, rather than inferred from a sample.</t>
+          <t>Earlier the claim rested on 23 probes. All 71 distinct endpoints observed in use were then probed with no credential: every one returned 403, none served data. The claim "no observed endpoint serves data to an unauthenticated caller" is now complete across the observed endpoint set, rather than inferred from a sample.</t>
         </is>
       </c>
     </row>
@@ -9337,7 +9362,7 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>- **The earlier coverage gap was self-inflicted, not a client dependency.** Six routes were recorded as blocked pending sample values for `:category`, `:invoiceId` and `:preEnquiryId`. All three were obtainable from the platform: - **Why it was missed:** the endpoint inventory is built from six sampled routes per persona, so screens never sampled — invoicing, the pre-enquiry list — contributed no endpoints, and their identifiers looked unobtainable when they were merely unvisited. The first harvest also ran while sessions were being rotated by a concurrent suite, which produced 401s that read as access failures. Neither was re-tested after the session handling was fixed.</t>
+          <t>The earlier coverage gap was self-inflicted, not a client dependency. Six routes were recorded as blocked pending sample values for :category, :invoiceId and :preEnquiryId. All three were obtainable from the platform: - Why it was missed: the endpoint inventory is built from six sampled routes per persona, so screens never sampled — invoicing, the pre-enquiry list — contributed no endpoints, and their identifiers looked unobtainable when they were merely unvisited. The first harvest also ran while sessions were being rotated by a concurrent suite, which produced 401s that read as access failures. Neither was re-tested after the session handling was fixed.</t>
         </is>
       </c>
     </row>
@@ -9359,7 +9384,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>- **No inter-application dependencies.** Every `required_apps` declaration is commented out, so the eight applications install independently of one another. Minimal external dependencies.** Only `outreach` declares any: `indiapins`, `gspread`, `google-auth` — all standard packages. The Google dependencies suggest a Sheets integration that may need credentials at runtime, relevant only to that feature.</t>
+          <t>No inter-application dependencies. Every required_apps declaration is commented out, so the eight applications install independently of one another. Minimal external dependencies. Only outreach declares any: indiapins, gspread, google-auth — all standard packages. The Google dependencies suggest a Sheets integration that may need credentials at runtime, relevant only to that feature.</t>
         </is>
       </c>
     </row>
@@ -9371,7 +9396,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>`Employee` is provided by ERPNext, resolving the earlier gap</t>
+          <t>Employee is provided by ERPNext, resolving the earlier gap</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -9381,7 +9406,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>- The authentication service queries an `Employee` doctype that none of the eight WeConnect applications defines. It is supplied by **ERPNext**, in its `Setup` module — confirmed on an installed instance by querying the doctype's owning module, not inferred. Frappe HR is not installed on the client's platform**, so the `HR-EMP-` identifier series comes from ERPNext's own naming configuration rather than from Frappe HR. An earlier note attributing it to Frappe HR was written before the installed-application list was read properly.</t>
+          <t>The authentication service queries an Employee doctype that none of the eight WeConnect applications defines. It is supplied by ERPNext, in its Setup module — confirmed on an installed instance by querying the doctype's owning module, not inferred. Frappe HR is not installed on the client's platform, so the HR-EMP- identifier series comes from ERPNext's own naming configuration rather than from Frappe HR. An earlier note attributing it to Frappe HR was written before the installed-application list was read properly.</t>
         </is>
       </c>
     </row>
@@ -9403,7 +9428,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>- **Check:** requested `DocType` metadata for 16 framework doctypes using the Skilling Manager account, both through `frappe.client.get_list` and the REST resource endpoint. Result:** **403 Permission Denied on every one.** An ordinary user cannot enumerate the schema, which is correct behaviour and the desired posture.</t>
+          <t>Check: requested DocType metadata for 16 framework doctypes using the Skilling Manager account, both through frappe.client.get_list and the REST resource endpoint. Result: 403 Permission Denied on every one. An ordinary user cannot enumerate the schema, which is correct behaviour and the desired posture.</t>
         </is>
       </c>
     </row>
@@ -9415,7 +9440,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>The login endpoint returns `api_key: null` on a repeat login</t>
+          <t>The login endpoint returns api_key: null on a repeat login</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -9425,7 +9450,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>- **Observed:** on a first login for an account, `authentication.api.auth.login` returns both `api_key` and `api_secret`. On a subsequent login for the same account it returned `api_key: null` with `api_secret` still populated. Why it matters to us:** any caller that re-authenticates and stores the returned pair will write a null key. This is adjacent to the session-rotation defect already recorded, where blind re-authentication rotated `api_secret` and invalidated in-flight sessions. Both point at the same underlying design: credential issue is stateful and a repeat login is not idempotent.</t>
+          <t>Observed: on a first login for an account, authentication.api.auth.login returns both api_key and api_secret. On a subsequent login for the same account it returned api_key: null with api_secret still populated. Why it matters to us: any caller that re-authenticates and stores the returned pair will write a null key. This is adjacent to the session-rotation defect already recorded, where blind re-authentication rotated api_secret and invalidated in-flight sessions. Both point at the same underlying design: credential issue is stateful and a repeat login is not idempotent.</t>
         </is>
       </c>
     </row>
@@ -9447,7 +9472,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>- Taken to size the Phase 2 synthetic dataset, using GET requests only, recording **counts and structure but never field values**. The resulting file contains zero record identifiers. - **Why it matters to the engagement:** a lifecycle test against one empty record is not the test the client needs. The synthetic dataset is scaled from these figures — roughly an order of magnitude smaller, preserving ratios and keeping list pagination (20 per page) exercised.</t>
+          <t>Taken to size the Phase 2 synthetic dataset, using GET requests only, recording counts and structure but never field values. The resulting file contains zero record identifiers. - Why it matters to the engagement: a lifecycle test against one empty record is not the test the client needs. The synthetic dataset is scaled from these figures — roughly an order of magnitude smaller, preserving ratios and keeping list pagination (20 per page) exercised.</t>
         </is>
       </c>
     </row>
@@ -9469,7 +9494,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>- **The platform does not use Frappe's `{"message": &lt;payload&gt;}` convention.** It returns its own envelope at the top level: ```json {"success_key": 1, "message": "Fetched Counselling successfully!", "data": [...], "count": 20, "total_pages": 41, "total_data_count": 810} ```</t>
+          <t>The platform does not use Frappe's {"message": &lt;payload&gt;} convention. It returns its own envelope at the top level: json {"success_key": 1, "message": "Fetched Counselling successfully!", "data": [...], "count": 20, "total_pages": 41, "total_data_count": 810}.</t>
         </is>
       </c>
     </row>
@@ -9491,7 +9516,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>- **Authorisation is by `User Permission` on `Lighthouse Centre`**, resolved at login into `permitted_centres`, with endpoints filtering against it. Frappe's role-permission system is not doing this work. Every doctype-level rule in source grants `System Manager` only. This is the root-cause class of the S1.** Where scope enforcement is a filter each endpoint must remember to apply, rather than a property the framework guarantees, a missing filter is not an anomaly. It is the expected failure mode. It also explains why sibling endpoints behave correctly while one does not: they are independent implementations, not a shared guarantee.</t>
+          <t>Authorisation is by User Permission on Lighthouse Centre, resolved at login into permitted_centres, with endpoints filtering against it. Frappe's role-permission system is not doing this work. Every doctype-level rule in source grants System Manager only. This is the root-cause class of the S1. Where scope enforcement is a filter each endpoint must remember to apply, rather than a property the framework guarantees, a missing filter is not an anomaly. It is the expected failure mode. It also explains why sibling endpoints behave correctly while one does not: they are independent implementations, not a shared guarantee.</t>
         </is>
       </c>
     </row>
@@ -9513,7 +9538,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>- **Probed on the isolated instance across all six fully-disjoint persona pairs**, for two operations — edit (`update_task`) and state change (`update_task_status`): Why this clean result means something.** Every probe carries two controls, because a refusal proves nothing on its own. An endpoint that is simply broken refuses everyone and reads as perfect access control:</t>
+          <t>Probed on the isolated instance across all six fully-disjoint persona pairs, for two operations — edit (update_task) and state change (update_task_status): Why this clean result means something. Every probe carries two controls, because a refusal proves nothing on its own. An endpoint that is simply broken refuses everyone and reads as perfect access control:</t>
         </is>
       </c>
     </row>
@@ -9535,7 +9560,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>- **Established on the isolated instance:** Frappe's `User Permission` restriction on `Lighthouse Centre` **correctly scopes** centre-linked records. A persona permitted for one centre, queried through the permission-respecting API (`get_list`), sees only that centre's records; a cross-centre write through the ordinary `.save()` path is refused with `PermissionError`. A method error was caught before it became a false finding.** An initial check used `frappe.get_all`, which **bypasses permissions by design**, and appeared to show a persona seeing all six centres' youth. Re-run with `frappe.get_list` (which enforces permissions) showed the correct scoping — 8 of 8 own-centre youth, none other</t>
+          <t>Established on the isolated instance: Frappe's User Permission restriction on Lighthouse Centre correctly scopes centre-linked records. A persona permitted for one centre, queried through the permission-respecting API (get_list), sees only that centre's records; a cross-centre write through the ordinary .save() path is refused with PermissionError. A method error was caught before it became a false finding. An initial check used frappe.get_all, which bypasses permissions by design, and appeared to show a persona seeing all six centres' youth. Re-run with frappe.get_list (which enforces permissions) showed the correct scoping — 8 of 8 own-centre youth, none other … (full detail in the findings register)</t>
         </is>
       </c>
     </row>
@@ -9547,7 +9572,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>`update_youth_status` cross-centre boundary holds</t>
+          <t>update_youth_status cross-centre boundary holds</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -9557,7 +9582,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>- Tested on a disjoint pair: `sp` (East/West) attempted to change the status of a youth owned by North via `youth_skilling.api.actions.update_youth_status`. Result: **refused**, `PermissionError`, youth status unchanged. Notable because the source looked unsafe: it performs a global `has_permission("Youth","write")` and then a `get_doc` with no centre check. The protection comes from `youth_doc.save()` re-applying User Permissions. This is the pattern the 30 truly-bypassed endpoints break by passing `ignore_permissions=True` to that same save.</t>
+          <t>Tested on a disjoint pair: sp (East/West) attempted to change the status of a youth owned by North via youth_skilling.api.actions.update_youth_status. Result: refused, PermissionError, youth status unchanged. Notable because the source looked unsafe: it performs a global has_permission("Youth","write") and then a get_doc with no centre check. The protection comes from youth_doc.save() re-applying User Permissions. This is the pattern the 30 truly-bypassed endpoints break by passing ignore_permissions=True to that same save.</t>
         </is>
       </c>
     </row>
@@ -9579,7 +9604,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>- **Verified end-to-end on the isolated instance**, as the owning persona through the API: 8 objects tested.** Create passes on 7 of 8 (Community Visit blocked on approval-workflow config). Read passes on all 7 created. Update passes on 6 of 7. The state-change column shows the richest picture: 2 clean passes, 1 confirmed defect (Enquiry Form typo), and a cluster of API-context 403s recorded separately as a reproducible discrepancy under investigation.</t>
+          <t>Verified end-to-end on the isolated instance, as the owning persona through the API: 8 objects tested. Create passes on 7 of 8 (Community Visit blocked on approval-workflow config). Read passes on all 7 created. Update passes on 6 of 7. The state-change column shows the richest picture: 2 clean passes, 1 confirmed defect (Enquiry Form typo), and a cluster of API-context 403s recorded separately as a reproducible discrepancy under investigation.</t>
         </is>
       </c>
     </row>
@@ -9601,7 +9626,7 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>- Creating a `Skilling Invoice` directly (to fixture the financial-endpoint test) failed with `pymysql OperationalError (1054): Unknown column 'skilling_batch' in 'WHERE'`, raised from within the invoice's own save path. The column `skilling_batch` exists on `Skilling Assessment Submission` (verified), so the failing query references it on a different table that lacks it — not located. Recorded as an observation, not a defect.** It may be that a synthetic invoice missing fields a real creation flow sets provokes a query with a bad value, rather than a universal bug. Invoices clearly exist in production, so the normal creation path works; ours did not, and the difference was not pursued to ro</t>
+          <t>Creating a Skilling Invoice directly (to fixture the financial-endpoint test) failed with pymysql OperationalError (1054): Unknown column 'skilling_batch' in 'WHERE', raised from within the invoice's own save path. The column skilling_batch exists on Skilling Assessment Submission (verified), so the failing query references it on a different table that lacks it — not located. Recorded as an observation, not a defect. It may be that a synthetic invoice missing fields a real creation flow sets provokes a query with a bad value, rather than a universal bug. Invoices clearly exist in production, so the normal creation path works; ours did not, and the difference was not pursued to root cause … (full detail in the findings register)</t>
         </is>
       </c>
     </row>
@@ -9623,7 +9648,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>- Creating a Community Visit auto-generates an Approval (via a doctype hook) whose category must have `ref_doc == "Community Visit"`. On a clean install no such category exists, so creation fails with "Invalid Approval Category for Document Type Community Visit." Configuring one did not immediately resolve it. The hook appears to select a category by a rule not yet traced. Recorded as the same class as the other config-not-in-repo findings:** the Community Visit flow depends on approval-category configuration that is production database state, absent from the repositories. Full lifecycle testing of Community Visit is deferred pending that configuration.</t>
+          <t>Creating a Community Visit auto-generates an Approval (via a doctype hook) whose category must have ref_doc == "Community Visit". On a clean install no such category exists, so creation fails with "Invalid Approval Category for Document Type Community Visit." Configuring one did not immediately resolve it. The hook appears to select a category by a rule not yet traced. Recorded as the same class as the other config-not-in-repo findings: the Community Visit flow depends on approval-category configuration that is production database state, absent from the repositories. Full lifecycle testing of Community Visit is deferred pending that configuration.</t>
         </is>
       </c>
     </row>
@@ -9645,7 +9670,7 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>- `youth_skilling.api.skilling_repository.add_course` validates **more than twenty required fields** before it will create a course — course_name, category, onboarding_date, screening flag, partner, training centre, certificate authority, lighthouse centre, QP code, education, eligibility remark, gender, age group, batch type, training mode, employment type, aligned job roles, durations, and more — several of them Links to other master records. Not a defect** — a course is a genuinely complex object. Recorded as a coverage note: driving its create through the API requires the full wizard payload, so full lifecycle automation of Course is materially more expensive than the simpler objects and</t>
+          <t>youth_skilling.api.skilling_repository.add_course validates more than twenty required fields before it will create a course — course_name, category, onboarding_date, screening flag, partner, training centre, certificate authority, lighthouse centre, QP code, education, eligibility remark, gender, age group, batch type, training mode, employment type, aligned job roles, durations, and more — several of them Links to other master records. Not a defect — a course is a genuinely complex object … (full detail in the findings register)</t>
         </is>
       </c>
     </row>
@@ -9667,7 +9692,7 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>- **Objects driven through their lifecycle (create/read/update/state):** Task, Pre Enquiry, Enquiry Form, Counselling, Approval, Follow Up, Skilling Issue (8th, Community Visit, blocked on approval config). Across personas fc, oc, ch, sp. Create succeeds on 7 of 8; read on 7; update on 6.** The state-change column is where the defects live: 2 clean, 1 confirmed defect (Enquiry typo), the verified API-403 cluster (S2).</t>
+          <t>Objects driven through their lifecycle (create/read/update/state): Task, Pre Enquiry, Enquiry Form, Counselling, Approval, Follow Up, Skilling Issue (8th, Community Visit, blocked on approval config). Across personas fc, oc, ch, sp. Create succeeds on 7 of 8; read on 7; update on 6. The state-change column is where the defects live: 2 clean, 1 confirmed defect (Enquiry typo), the verified API-403 cluster (S2).</t>
         </is>
       </c>
     </row>
@@ -9689,7 +9714,7 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>- **Method.** Six mutation endpoints across four personas were fed (a) an empty payload and (b) a well-formed payload carrying invalid values — nonexistent link references, bad enum values, an end-date before the start-date. `data/validation-probe-results.json` has the table. - **The clean result — validation itself works.** **No endpoint accepted invalid data** (zero false-OK). Bad enum values, nonexistent references and impossible dates were all refused. Invalid data does not get written. This is the property that matters most, and it holds.</t>
+          <t>Method. Six mutation endpoints across four personas were fed (a) an empty payload and (b) a well-formed payload carrying invalid values — nonexistent link references, bad enum values, an end-date before the start-date. data/validation-probe-results.json has the table. - The clean result — validation itself works. No endpoint accepted invalid data (zero false-OK). Bad enum values, nonexistent references and impossible dates were all refused. Invalid data does not get written. This is the property that matters most, and it holds.</t>
         </is>
       </c>
     </row>
@@ -9711,7 +9736,7 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>- **Tested:** `update_youth_status` called with a list of two IDs — one valid (a North youth the FC persona owns) and one nonexistent — and a status change. Result:** the endpoint returned HTTP 400 "Invalid id" and **the valid youth's status was unchanged** — it validated the entire batch before applying any change, rather than mutating the valid record and then failing on the invalid one.</t>
+          <t>Tested: update_youth_status called with a list of two IDs — one valid (a North youth the FC persona owns) and one nonexistent — and a status change. Result: the endpoint returned HTTP 400 "Invalid id" and the valid youth's status was unchanged — it validated the entire batch before applying any change, rather than mutating the valid record and then failing on the invalid one.</t>
         </is>
       </c>
     </row>
@@ -9733,7 +9758,7 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>- Built `utils/auto-create-probe.mjs`, which drives a create endpoint by iterating call -&gt; read the error -&gt; satisfy it -&gt; retry, resolving required fields, invalid links (by querying the database) and enum constraints automatically. It extended create coverage** to Registration Form B and re-confirmed Task, Skilling Issue and Follow Up without hand-built payloads.</t>
+          <t>Built utils/auto-create-probe.mjs, which drives a create endpoint by iterating call -&gt; read the error -&gt; satisfy it -&gt; retry, resolving required fields, invalid links (by querying the database) and enum constraints automatically. It extended create coverage to Registration Form B and re-confirmed Task, Skilling Issue and Follow Up without hand-built payloads.</t>
         </is>
       </c>
     </row>
@@ -9745,7 +9770,7 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>A PostgreSQL data dump is stored in the `data-pipeline-dashboard` repository</t>
+          <t>A PostgreSQL data dump is stored in the data-pipeline-dashboard repository</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -9755,7 +9780,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Not raised as a defect.** Recorded for completeness because the file was examined during the review of the foundation's GitHub organisation, and because a reader of the register may otherwise wonder whether it was missed. - **Where:** `Lighthouse-Communities-Foundation/data-pipeline-dashboard`, `lcf_data.sql`, on the default branch. The repository is **private**.</t>
+          <t>Not raised as a defect. Recorded for completeness because the file was examined during the review of the foundation's GitHub organisation, and because a reader of the register may otherwise wonder whether it was missed. - Where: Lighthouse-Communities-Foundation/data-pipeline-dashboard, lcf_data.sql, on the default branch. The repository is private.</t>
         </is>
       </c>
     </row>
@@ -9777,7 +9802,7 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>This engagement's security testing grew out of functional QA rather than from a security standard, so its coverage was mapped against the OWASP API Security Top 10 after the fact. The mapping is recorded here so that what was and was not examined is explicit. Follow-up (2026-09-22): the four untested categories have since been examined**, together with SQL injection and file upload. API7 came back clean; API3, API4 and API6 each produced findings, recorded above. Injection is clean (all 339 raw SQL calls taint-analysed). The only remaining partial areas are a full mass-assignment sweep across every `data`-accepting endpoint, and CORS configuration.</t>
+          <t>This engagement's security testing grew out of functional QA rather than from a security standard, so its coverage was mapped against the OWASP API Security Top 10 after the fact. The mapping is recorded here so that what was and was not examined is explicit. Follow-up (2026-09-22): the four untested categories have since been examined, together with SQL injection and file upload. API7 came back clean; API3, API4 and API6 each produced findings, recorded above. Injection is clean (all 339 raw SQL calls taint-analysed). The only remaining partial areas are a full mass-assignment sweep across every data-accepting endpoint, and CORS configuration.</t>
         </is>
       </c>
     </row>
@@ -9799,7 +9824,7 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Assessed in response to the OWASP/CWE injection category, which had not been examined systematically. The result is a clean one, recorded here so that what was checked is explicit. - **Method.** Every `frappe.db.sql()` call in the eight applications was located by static analysis (339 in total), and each was classified by what it interpolates into the SQL string: a locally-built clause fragment, a value derived from the ORM or the server, or a value reaching the string directly from a request parameter.</t>
+          <t>Assessed in response to the OWASP/CWE injection category, which had not been examined systematically. The result is a clean one, recorded here so that what was checked is explicit. - Method. Every frappe.db.sql() call in the eight applications was located by static analysis (339 in total), and each was classified by what it interpolates into the SQL string: a locally-built clause fragment, a value derived from the ORM or the server, or a value reaching the string directly from a request parameter.</t>
         </is>
       </c>
     </row>
@@ -9821,7 +9846,7 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Completes the API3 category. This entry replaces an earlier version that reported 28 sites with 22 filtered and 6 not. Re-running the analysis with two faults removed changed the answer, and the earlier figures should not be relied on. 1. **Commented-out code was counted.** `outreach/apis/pec/form.py` contains a large block of dead code around line 518 in which a `doc.update(data)` and a `save(ignore_permissions=True)` appear. Every line is commented. It is not reachable and should never have been in the count. 2. **A denylist was read as a filter.** Several handlers call `remove_keys_from_dict(data, keys_to_remove)` or `data.pop(...)` before the write. That removes the keys the handler has </t>
+          <t>Completes the API3 category. This entry replaces an earlier version that reported 28 sites with 22 filtered and 6 not. Re-running the analysis with two faults removed changed the answer, and the earlier figures should not be relied on. 1. Commented-out code was counted. outreach/apis/pec/form.py contains a large block of dead code around line 518 in which a doc.update(data) and a save(ignore_permissions=True) appear. Every line is commented. It is not reachable and should never have been in the count. 2. A denylist was read as a filter. Several handlers call remove_keys_from_dict(data, keys_to_remove) or data.pop(...) before the write … (full detail in the findings register)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add what-we-need-from-you block to tracker and correct date count
</commit_message>
<xml_diff>
--- a/tracker/WeConnect-QA-Bug-Tracker.xlsx
+++ b/tracker/WeConnect-QA-Bug-Tracker.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -728,7 +728,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Populated for the 15 defects where our register records a date. We did not record a date against every finding, and we have not invented them. Use the Phase column instead for rough sequencing.</t>
+          <t>Populated for the 14 defects where our register records a date. We did not record a date against every finding, and we have not invented them. Use the Phase column instead for rough sequencing.</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>RE-CHECKING A FIX</t>
+          <t>WHAT WE NEED FROM YOU — nothing in this sheet is blocked on us</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr"/>
@@ -771,22 +771,82 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>23 of the 79 can be re-checked mechanically</t>
+          <t>1. Fix these four now</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Run: node verify/run.mjs --only &lt;Bug ID&gt; — no installation, read-only by default. The Re-check Command column gives the exact line.</t>
+          <t>WC-088, WC-068, WC-023, WC-121. Minutes of work each. They are the four a reader of this sheet could act on, so they should not wait for a planning cycle.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>2. Sign the characterisation document</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Part 1 of docs/CHARACTERISATION.md, about ten minutes. Confirm seven answers we worked out ourselves, acknowledge six, and answer two: whether there is an escrow arrangement for fintoo_analytics_bridge, and whether each role has the right screens. Until that is signed we cannot assert what correct behaviour is, so functional testing and regression closure both wait on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>3. Decide on BrowserStack</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>See docs/BROWSERSTACK-RECOMMENDATION.md. One decision; it affects Phase 3 scope and cost, not the schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Everything else</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3 cross-browser execution and CI can start without any of the above, because they run the existing suites.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>RE-CHECKING A FIX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>23 of the 79 can be re-checked mechanically</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Run: node verify/run.mjs --only &lt;Bug ID&gt; — no installation, read-only by default. The Re-check Command column gives the exact line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t>The rest</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Re-check by following the Steps to Reproduce column.</t>
         </is>

</xml_diff>

<commit_message>
Rewrite tracker notes as reference documentation
</commit_message>
<xml_diff>
--- a/tracker/WeConnect-QA-Bug-Tracker.xlsx
+++ b/tracker/WeConnect-QA-Bug-Tracker.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Phases 1 and 2: read-only testing and transactional testing</t>
+          <t>Phases 1 and 2 — read-only testing and transactional testing</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>findings/findings-log.md in the QA repository. Every row here carries its Bug ID so the two can be reconciled.</t>
+          <t>findings/findings-log.md in the QA repository. Each row carries its Bug ID, so any entry here can be traced to its full write-up.</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>TABS</t>
+          <t>Contents</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr"/>
@@ -608,7 +608,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>79 defects. One row each, with the five fields you asked for plus severity, priority and re-check instructions.</t>
+          <t>79 defects, one per row, ordered by priority.</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Previous Day / Today progress, one row per working day, taken from our dated working record.</t>
+          <t>Progress by working day, with the previous day's work shown beside each day's.</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Counts by severity, priority and area. All figures are formulas reading the Bugs tab, so they update if you edit it.</t>
+          <t>Counts by severity, priority, area and status. Figures are formulas over the Bugs tab and update when it is edited.</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>40 informational records. These are NOT defects — they are context we recorded. Kept separate so they do not inflate the bug count.</t>
+          <t>40 informational records. These are not defects and cannot be closed; they are held separately so they do not affect the defect count.</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>COLUMNS YOU FILL IN — shaded pale yellow</t>
+          <t>Column reference</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr"/>
@@ -663,192 +663,220 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Bug ID</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>We have set every row to Open. Change it as work proceeds.</t>
+          <t>Stable identifier. Does not change if severity or ordering changes.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Assigned To</t>
+          <t>Severity</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Blank. Yours to allocate.</t>
+          <t>S1 Blocker, S2 Critical, S3 Major, S4 Minor, on the ISTQB scale.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Previous Day Status / Today's Status</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Seeded with what we know as of the last re-check. Maintain these daily.</t>
+          <t>P1 to P4. Weighs the cost of the fix against the cost of leaving it, so it differs from severity in both directions.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Target Fix Date</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Blank. Yours to set.</t>
+          <t>Where the defect was observed: UAT/dev read-only, the isolated stack with synthetic data, or source review.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-      <c r="B20" s="3" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Steps to Reproduce</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Numbered steps. Entries marked as code review or inspection have no runtime reproduction and say so.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>WHAT WE COULD NOT FILL IN, AND WHY</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Derived from the defect class. The characterisation document is unsigned, so for behavioural questions this is our reading rather than an agreed specification.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Date Reported</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Populated for the 14 defects where our register records a date. We did not record a date against every finding, and we have not invented them. Use the Phase column instead for rough sequencing.</t>
+          <t>What was observed, quoted from the register.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Screenshots</t>
+          <t>Attachment / Screenshot Reference</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Images exist for 5 defects — the ones with a visible screen that failed. The other 74 are API or source-code findings with nothing to photograph. For those the Attachment column points at the probe output, the script that reproduces it, or a one-line re-check command, which is stronger evidence than a screenshot.</t>
+          <t>Screen captures for 5 defects, being those with a visible screen that failed. The remainder cite probe output, the script that reproduces the defect, or a re-check command.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Expected Result</t>
+          <t>How Verified</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Derived from the defect class, not from a signed specification. The characterisation document is not yet signed, so for a handful of behavioural questions 'expected' is still our reading rather than your agreement.</t>
+          <t>How the defect was established, as recorded in the register.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
-      <c r="B25" s="3" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Date Reported</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Recorded for 14 of 79. Per-finding dates were not captured for the remainder; the Phase column gives approximate sequence.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>WHAT WE NEED FROM YOU — nothing in this sheet is blocked on us</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Re-check Command</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Present for the 23 defects that can be verified mechanically.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>1. Fix these four now</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>WC-088, WC-068, WC-023, WC-121. Minutes of work each. They are the four a reader of this sheet could act on, so they should not wait for a planning cycle.</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2. Sign the characterisation document</t>
+          <t>Maintained by Lighthouse</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Part 1 of docs/CHARACTERISATION.md, about ten minutes. Confirm seven answers we worked out ourselves, acknowledge six, and answer two: whether there is an escrow arrangement for fintoo_analytics_bridge, and whether each role has the right screens. Until that is signed we cannot assert what correct behaviour is, so functional testing and regression closure both wait on it.</t>
+          <t>Shaded pale yellow: Status, Assigned To, Target Fix Date, Previous Day Status, Today's Status. Status is set to Open throughout and carries a dropdown.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>3. Decide on BrowserStack</t>
+          <t>Re-checking a fix</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>See docs/BROWSERSTACK-RECOMMENDATION.md. One decision; it affects Phase 3 scope and cost, not the schedule.</t>
+          <t>For the 23 with a Re-check Command, run: node verify/run.mjs --only &lt;Bug ID&gt;. It requires Node, installs nothing, and issues read-only requests by default. For the remainder, follow the Steps to Reproduce column.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Everything else</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Phase 3 cross-browser execution and CI can start without any of the above, because they run the existing suites.</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Outstanding items</t>
+        </is>
+      </c>
       <c r="B31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>RE-CHECKING A FIX</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Immediate fixes</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>WC-088, WC-068, WC-023 and WC-121 are each a few minutes of work and require no planning cycle.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>23 of the 79 can be re-checked mechanically</t>
+          <t>Characterisation sign-off</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Run: node verify/run.mjs --only &lt;Bug ID&gt; — no installation, read-only by default. The Re-check Command column gives the exact line.</t>
+          <t>Part 1 of docs/CHARACTERISATION.md. Seven answers to confirm, six to acknowledge, two to answer. Functional-correctness testing and regression closure depend on it.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>The rest</t>
+          <t>BrowserStack capacity</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Re-check by following the Steps to Reproduce column.</t>
+          <t>One decision, set out in docs/BROWSERSTACK-RECOMMENDATION.md. Affects Phase 3 scope and cost rather than schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Independent of the above</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3 cross-browser execution and continuous integration run the existing suites and need no decision.</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1057,7 @@
       <c r="H2" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as an authenticated staff account and take the API credential from the login response.
-2. Identify a record owned by a centre this account is NOT permitted for.
+2. Identify a record owned by a centre this account is not permitted for.
 3. Call facilitator_and_counsellor.api.counselling.list.get_counselling_list against that record.
 4. Read the response, then read the record back from the database — the response alone is not proof.</t>
         </is>
@@ -1056,7 +1084,7 @@
       </c>
       <c r="M2" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N2" s="7" t="inlineStr">
@@ -1126,7 +1154,7 @@
       <c r="H3" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as Skilling Partner and take the API credential from the login response.
-2. Identify a record owned by a centre this account is NOT permitted for.
+2. Identify a record owned by a centre this account is not permitted for.
 3. Call youth_skilling.api.batch_management.close_batch(batch_id, short_remarks) against that record.
 4. Read the response, then read the record back from the database — the response alone is not proof.</t>
         </is>
@@ -1153,7 +1181,7 @@
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime, end-to-end breach</t>
+          <t>Verified — runtime, end-to-end breach</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr"/>
@@ -1219,7 +1247,7 @@
       <c r="H4" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as Skilling Partner and take the API credential from the login response.
-2. Identify a record owned by a centre this account is NOT permitted for.
+2. Identify a record owned by a centre this account is not permitted for.
 3. Call youth_skilling.api.invoice.raise_invoice(invoice_id, batch_id, center, installment, ...) against that record.
 4. Read the response, then read the record back from the database — the response alone is not proof.</t>
         </is>
@@ -1246,7 +1274,7 @@
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime, end-to-end breach</t>
+          <t>Verified — runtime, end-to-end breach</t>
         </is>
       </c>
       <c r="N4" s="7" t="inlineStr"/>
@@ -1338,7 +1366,7 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — observed at first contact</t>
+          <t>Verified — observed at first contact</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr"/>
@@ -1430,7 +1458,7 @@
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — ESCALATED 2026-09-19</t>
+          <t>Verified — escalated 2026-09-19</t>
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr">
@@ -1526,7 +1554,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr"/>
@@ -1619,7 +1647,7 @@
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N8" s="7" t="inlineStr"/>
@@ -1711,7 +1739,7 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — ROOT CAUSE, corrects an earlier classification</t>
+          <t>Verified — root cause, corrects an earlier classification</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr"/>
@@ -1803,7 +1831,7 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr"/>
@@ -1895,7 +1923,7 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr"/>
@@ -1987,7 +2015,7 @@
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime blocks it</t>
+          <t>Verified — runtime blocks it</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr"/>
@@ -2079,7 +2107,7 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr"/>
@@ -2171,7 +2199,7 @@
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source + 36/36 confirmed at runtime</t>
+          <t>Verified — source + 36/36 confirmed at runtime</t>
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr"/>
@@ -2237,7 +2265,7 @@
       <c r="H15" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as an authenticated staff account and take the API credential from the login response.
-2. Identify a record owned by a centre this account is NOT permitted for.
+2. Identify a record owned by a centre this account is not permitted for.
 3. Call youth_skilling.api.invoice.raise_invoice(invoice_id, batch_id, center, installment, ...) against that record.
 4. Read the response, then read the record back from the database — the response alone is not proof.</t>
         </is>
@@ -2264,7 +2292,7 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source; runtime blocked by fixture</t>
+          <t>Verified — source; runtime blocked by fixture</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr"/>
@@ -2356,7 +2384,7 @@
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="N16" s="7" t="inlineStr">
@@ -2426,7 +2454,7 @@
       <c r="H17" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as an authenticated staff account and take the API credential from the login response.
-2. Identify a record owned by a centre this account is NOT permitted for.
+2. Identify a record owned by a centre this account is not permitted for.
 3. Call the 45 scoping sites across 26 files (evidence/authz-audit.json) against that record.
 4. Read the response, then read the record back from the database — the response alone is not proof.</t>
         </is>
@@ -2453,7 +2481,7 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source, 45 sites; one instance confirmed exploited on the live platform, runtime read-only</t>
+          <t>Verified — source, 45 sites; one instance confirmed exploited on the live platform, runtime read-only</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr"/>
@@ -2545,7 +2573,7 @@
       </c>
       <c r="M18" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime, isolated instance</t>
+          <t>Verified — runtime, isolated instance</t>
         </is>
       </c>
       <c r="N18" s="7" t="inlineStr"/>
@@ -2637,7 +2665,7 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — observed at first contact</t>
+          <t>Verified — observed at first contact</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr"/>
@@ -2725,7 +2753,7 @@
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N20" s="7" t="inlineStr">
@@ -2818,7 +2846,7 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr"/>
@@ -2906,7 +2934,7 @@
       </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — three consecutive executions, 2026-09-19</t>
+          <t>Verified — three consecutive executions, 2026-09-19</t>
         </is>
       </c>
       <c r="N22" s="7" t="inlineStr">
@@ -2998,7 +3026,7 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — new</t>
+          <t>Verified — new</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr"/>
@@ -3086,7 +3114,7 @@
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N24" s="7" t="inlineStr">
@@ -3178,7 +3206,7 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
@@ -3270,7 +3298,7 @@
       </c>
       <c r="M26" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N26" s="7" t="inlineStr"/>
@@ -3358,7 +3386,7 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — dose-response</t>
+          <t>Verified — dose-response</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr"/>
@@ -3447,7 +3475,7 @@
       </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — CORRECTED 2026-09-20</t>
+          <t>Verified — corrected 2026-09-20</t>
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr">
@@ -3540,7 +3568,7 @@
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr"/>
@@ -3629,7 +3657,7 @@
       </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N30" s="7" t="inlineStr"/>
@@ -3718,7 +3746,7 @@
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr"/>
@@ -3806,7 +3834,7 @@
       </c>
       <c r="M32" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="N32" s="7" t="inlineStr"/>
@@ -3895,7 +3923,7 @@
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime, root-caused</t>
+          <t>Verified — runtime, root-caused</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr"/>
@@ -3983,7 +4011,7 @@
       </c>
       <c r="M34" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source, all 9 frontend repositories; hosts confirmed distinct at runtime via DNS and probe</t>
+          <t>Verified — source, all 9 frontend repositories; hosts confirmed distinct at runtime via DNS and probe</t>
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr"/>
@@ -4071,7 +4099,7 @@
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source, auth application routing table + backend + repository listing</t>
+          <t>Verified — source, auth application routing table + backend + repository listing</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr"/>
@@ -4160,7 +4188,7 @@
       </c>
       <c r="M36" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source + clean install, 2026-09-20</t>
+          <t>Verified — source + clean install, 2026-09-20</t>
         </is>
       </c>
       <c r="N36" s="7" t="inlineStr">
@@ -4253,7 +4281,7 @@
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — live, read-only</t>
+          <t>Verified — live, read-only</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr"/>
@@ -4346,7 +4374,7 @@
       </c>
       <c r="M38" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="N38" s="7" t="inlineStr"/>
@@ -4434,7 +4462,7 @@
       </c>
       <c r="M39" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — reproduced against the isolated stack</t>
+          <t>Verified — reproduced against the isolated stack</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr"/>
@@ -4526,7 +4554,7 @@
       </c>
       <c r="M40" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — reproduced against the isolated stack</t>
+          <t>Verified — reproduced against the isolated stack</t>
         </is>
       </c>
       <c r="N40" s="7" t="inlineStr"/>
@@ -4619,7 +4647,7 @@
       </c>
       <c r="M41" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — reproduced against the isolated stack</t>
+          <t>Verified — reproduced against the isolated stack</t>
         </is>
       </c>
       <c r="N41" s="7" t="inlineStr"/>
@@ -4712,7 +4740,7 @@
       </c>
       <c r="M42" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="N42" s="7" t="inlineStr">
@@ -4804,7 +4832,7 @@
       </c>
       <c r="M43" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N43" s="7" t="inlineStr"/>
@@ -4892,7 +4920,7 @@
       </c>
       <c r="M44" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source</t>
+          <t>Verified — source</t>
         </is>
       </c>
       <c r="N44" s="7" t="inlineStr"/>
@@ -4980,7 +5008,7 @@
       </c>
       <c r="M45" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source</t>
+          <t>Verified — source</t>
         </is>
       </c>
       <c r="N45" s="7" t="inlineStr"/>
@@ -5068,7 +5096,7 @@
       </c>
       <c r="M46" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr"/>
@@ -5156,7 +5184,7 @@
       </c>
       <c r="M47" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime, three disjoint personas</t>
+          <t>Verified — runtime, three disjoint personas</t>
         </is>
       </c>
       <c r="N47" s="7" t="inlineStr"/>
@@ -5245,7 +5273,7 @@
       </c>
       <c r="M48" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — System Settings, isolated instance built from the client's own configuration path</t>
+          <t>Verified — System Settings, isolated instance built from the client's own configuration path</t>
         </is>
       </c>
       <c r="N48" s="7" t="inlineStr"/>
@@ -5338,7 +5366,7 @@
       </c>
       <c r="M49" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — observed against the live backend</t>
+          <t>Verified — observed against the live backend</t>
         </is>
       </c>
       <c r="N49" s="7" t="inlineStr"/>
@@ -5430,7 +5458,7 @@
       </c>
       <c r="M50" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — reproduced against the isolated stack</t>
+          <t>Verified — reproduced against the isolated stack</t>
         </is>
       </c>
       <c r="N50" s="7" t="inlineStr"/>
@@ -5518,7 +5546,7 @@
       </c>
       <c r="M51" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="N51" s="7" t="inlineStr"/>
@@ -5606,7 +5634,7 @@
       </c>
       <c r="M52" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="N52" s="7" t="inlineStr"/>
@@ -5694,7 +5722,7 @@
       </c>
       <c r="M53" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N53" s="7" t="inlineStr">
@@ -5786,7 +5814,7 @@
       </c>
       <c r="M54" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N54" s="7" t="inlineStr">
@@ -5878,7 +5906,7 @@
       </c>
       <c r="M55" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N55" s="7" t="inlineStr"/>
@@ -5966,7 +5994,7 @@
       </c>
       <c r="M56" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N56" s="7" t="inlineStr"/>
@@ -6054,7 +6082,7 @@
       </c>
       <c r="M57" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N57" s="7" t="inlineStr"/>
@@ -6142,7 +6170,7 @@
       </c>
       <c r="M58" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N58" s="7" t="inlineStr"/>
@@ -6231,7 +6259,7 @@
       </c>
       <c r="M59" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N59" s="7" t="inlineStr"/>
@@ -6320,7 +6348,7 @@
       </c>
       <c r="M60" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N60" s="7" t="inlineStr"/>
@@ -6409,7 +6437,7 @@
       </c>
       <c r="M61" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N61" s="7" t="inlineStr">
@@ -6501,7 +6529,7 @@
       </c>
       <c r="M62" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N62" s="7" t="inlineStr"/>
@@ -6589,7 +6617,7 @@
       </c>
       <c r="M63" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N63" s="7" t="inlineStr"/>
@@ -6677,7 +6705,7 @@
       </c>
       <c r="M64" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N64" s="7" t="inlineStr">
@@ -6769,7 +6797,7 @@
       </c>
       <c r="M65" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N65" s="7" t="inlineStr"/>
@@ -6857,7 +6885,7 @@
       </c>
       <c r="M66" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime, pattern</t>
+          <t>Verified — runtime, pattern</t>
         </is>
       </c>
       <c r="N66" s="7" t="inlineStr"/>
@@ -6945,7 +6973,7 @@
       </c>
       <c r="M67" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — corrects the earlier observation</t>
+          <t>Verified — corrects the earlier observation</t>
         </is>
       </c>
       <c r="N67" s="7" t="inlineStr"/>
@@ -7033,7 +7061,7 @@
       </c>
       <c r="M68" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="N68" s="7" t="inlineStr"/>
@@ -7121,7 +7149,7 @@
       </c>
       <c r="M69" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="N69" s="7" t="inlineStr"/>
@@ -7210,7 +7238,7 @@
       </c>
       <c r="M70" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source</t>
+          <t>Verified — source</t>
         </is>
       </c>
       <c r="N70" s="7" t="inlineStr"/>
@@ -7298,7 +7326,7 @@
       </c>
       <c r="M71" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime, isolated instance</t>
+          <t>Verified — runtime, isolated instance</t>
         </is>
       </c>
       <c r="N71" s="7" t="inlineStr"/>
@@ -7387,7 +7415,7 @@
       </c>
       <c r="M72" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="N72" s="7" t="inlineStr"/>
@@ -7476,7 +7504,7 @@
       </c>
       <c r="M73" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="N73" s="7" t="inlineStr"/>
@@ -7565,7 +7593,7 @@
       </c>
       <c r="M74" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="N74" s="7" t="inlineStr"/>
@@ -7654,7 +7682,7 @@
       </c>
       <c r="M75" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="N75" s="7" t="inlineStr"/>
@@ -7743,7 +7771,7 @@
       </c>
       <c r="M76" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="N76" s="7" t="inlineStr"/>
@@ -7831,7 +7859,7 @@
       </c>
       <c r="M77" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N77" s="7" t="inlineStr"/>
@@ -7920,7 +7948,7 @@
       </c>
       <c r="M78" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N78" s="7" t="inlineStr"/>
@@ -8009,7 +8037,7 @@
       </c>
       <c r="M79" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N79" s="7" t="inlineStr"/>
@@ -8097,7 +8125,7 @@
       </c>
       <c r="M80" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source</t>
+          <t>Verified — source</t>
         </is>
       </c>
       <c r="N80" s="7" t="inlineStr"/>
@@ -9043,7 +9071,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -9087,7 +9115,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -9109,7 +9137,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -9131,7 +9159,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -9175,7 +9203,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -9197,7 +9225,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -9219,7 +9247,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -9241,7 +9269,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -9263,7 +9291,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>(untagged)</t>
+          <t>Not recorded</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -9285,7 +9313,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — clean result</t>
+          <t>Verified — clean result</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -9351,7 +9379,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -9373,7 +9401,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -9395,7 +9423,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — clean result</t>
+          <t>Verified — clean result</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -9417,7 +9445,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -9439,7 +9467,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -9461,7 +9489,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -9483,7 +9511,7 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — clean result</t>
+          <t>Verified — clean result</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -9505,7 +9533,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — reproducible in isolation</t>
+          <t>Verified — reproducible in isolation</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -9527,7 +9555,7 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — no values recorded</t>
+          <t>Verified — no values recorded</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -9549,7 +9577,7 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -9571,7 +9599,7 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -9593,7 +9621,7 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — clean result</t>
+          <t>Verified — clean result</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -9615,7 +9643,7 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime, corrects a query-method error</t>
+          <t>Verified — runtime, corrects a query-method error</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -9637,7 +9665,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime, clean result</t>
+          <t>Verified — runtime, clean result</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -9659,7 +9687,7 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -9747,7 +9775,7 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -9769,7 +9797,7 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — runtime</t>
+          <t>Verified — runtime</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -9791,7 +9819,7 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — clean result</t>
+          <t>Verified — clean result</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -9813,7 +9841,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -9835,7 +9863,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — archive TOC and schema; confirmed intentional by the QA lead</t>
+          <t>Verified — archive TOC and schema; confirmed intentional by the QA lead</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
@@ -9879,7 +9907,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source, taint analysis of all 339 raw SQL calls</t>
+          <t>Verified — source, taint analysis of all 339 raw SQL calls</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -9901,7 +9929,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>VERIFIED — source analysis, re-run 2026-09-25</t>
+          <t>Verified — source analysis, re-run 2026-09-25</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Correct reproduction steps for eight defects
</commit_message>
<xml_diff>
--- a/tracker/WeConnect-QA-Bug-Tracker.xlsx
+++ b/tracker/WeConnect-QA-Bug-Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bugs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Daily Report" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Observations" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Report" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bugs'!$A$1:$T$80</definedName>
@@ -1431,9 +1431,10 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>1. Sign in as an authenticated staff account.
-2. Call youth_skilling.api.screening.screening_schedule_list omitting a required argument, or with an argument of the wrong type.
-3. Read the HTTP status and the response body.</t>
+          <t>1. No sign-in needed.
+2. Trigger any API error — for example call an endpoint without a credential, or with an unknown identifier.
+3. Read the response body and look for an exc field carrying a Python traceback and server filesystem paths.
+4. Fastest route: node verify/run.mjs --only WC-023</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
@@ -1713,8 +1714,9 @@
       <c r="H9" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as Facilitator and Counsellor.
-2. Call /fc/badge-table omitting a required argument, or with an argument of the wrong type.
-3. Read the HTTP status and the response body.</t>
+2. Paste /fc/badge-table into the address bar and load it directly, rather than navigating to it inside the app.
+3. The screen renders blank. Open the browser console and read the exception, which names the property read from a null navigation state.
+4. Repeat from inside the app by clicking through to the same screen; it renders.</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -2357,9 +2359,10 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>1. Sign in as an authenticated staff account.
-2. Call outreach/apis/enquiry_form/form.py:38 and outreach/apis/enquiry.py:248 — update_status(ids, document, data) omitting a required argument, or with an argument of the wrong type.
-3. Read the HTTP status and the response body.</t>
+          <t>1. Sign in as an account permitted for the Enquiry Form screen.
+2. Change the status of any Enquiry Form through the API, with a valid payload.
+3. The call returns HTTP 500 UnboundLocalError. It fails on every call, not only on malformed input, because the handler reads a variable that was never assigned.
+4. The same defect is present at two sites: outreach/apis/enquiry_form/form.py:38 and outreach/apis/enquiry.py:248.</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
@@ -3088,8 +3091,8 @@
       <c r="H24" s="7" t="inlineStr">
         <is>
           <t>1. Sign in as Skilling Youth Coordinator.
-2. Call youth_skilling.api.curriculum.curriculum_list omitting a required argument, or with an argument of the wrong type.
-3. Read the HTTP status and the response body.</t>
+2. Open the curriculum screen, or call youth_skilling.api.curriculum.curriculum_list directly with valid arguments.
+3. Read the HTTP status. The call fails on a correctly formed request, not only on a malformed one.</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
@@ -3807,9 +3810,9 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>1. Sign in as an authenticated staff account.
-2. Call facilitator_and_counsellor.api.counselling.actions.mark_as_dropoff omitting a required argument, or with an argument of the wrong type.
-3. Read the HTTP status and the response body.</t>
+          <t>1. Sign in as Administrator, the highest-privilege account available.
+2. Call the affected endpoint over HTTP with valid arguments.
+3. The call returns 403 even for Administrator, while the same function succeeds when invoked directly on the server.</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
@@ -6055,9 +6058,9 @@
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>1. Sign in as an authenticated staff account.
-2. Call authentication.api.auth.login omitting a required argument, or with an argument of the wrong type.
-3. Read the HTTP status and the response body.</t>
+          <t>1. Sign in as each of the six personas in turn.
+2. Read permitted_courses in each login response.
+3. Compare the type across accounts: three return an array, three return the string NA.</t>
         </is>
       </c>
       <c r="I57" s="7" t="inlineStr">
@@ -6590,9 +6593,9 @@
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>1. Sign in as an authenticated staff account.
-2. Call weconnect-backend-batch-management, batch_management/fixtures/custom_field.json — adds custom_abbr ("ABBR") to Cost Center as fieldtype: Data, reqd: 1, with no default omitting a required argument, or with an argument of the wrong type.
-3. Read the HTTP status and the response body.</t>
+          <t>1. On a clean install built from the repositories, attempt to create an ERPNext Company.
+2. Submit the form with all mandatory fields completed.
+3. Creation fails on the custom_abbr custom field, which has no default.</t>
         </is>
       </c>
       <c r="I63" s="7" t="inlineStr">
@@ -6946,9 +6949,9 @@
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>1. Sign in as an authenticated staff account.
-2. Call the Skilling Invoice doctype's validate() method omitting a required argument, or with an argument of the wrong type.
-3. Read the HTTP status and the response body.</t>
+          <t>1. Create or save a Skilling Invoice on an install built from the repositories.
+2. The doctype's validate() method runs on save and queries a column that is not present in the schema.
+3. The save fails with a SQL error naming the missing column.</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Set tracker font to Times New Roman
</commit_message>
<xml_diff>
--- a/tracker/WeConnect-QA-Bug-Tracker.xlsx
+++ b/tracker/WeConnect-QA-Bug-Tracker.xlsx
@@ -33,28 +33,28 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <b val="1"/>
       <color rgb="003A2E6E"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <color rgb="00444444"/>
       <sz val="10"/>
     </font>

</xml_diff>

<commit_message>
Re-test against client fixes 2026-10-08: record verified-fixed, partial, still-present per finding
</commit_message>
<xml_diff>
--- a/tracker/WeConnect-QA-Bug-Tracker.xlsx
+++ b/tracker/WeConnect-QA-Bug-Tracker.xlsx
@@ -1307,7 +1307,7 @@
       </c>
       <c r="V3" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present — close_batch has no centre/permission check in current source</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="V4" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Possibly fixed — new centre-scope layer in invoice.py; unconfirmed (write path, SP account not provisioned)</t>
         </is>
       </c>
       <c r="W4" s="7" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="V6" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present on api-dev 2026-10-08</t>
         </is>
       </c>
       <c r="W6" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="V10" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Partially fixed — youth_skilling specs now require auth; batch_management spec still public</t>
         </is>
       </c>
       <c r="W10" s="7" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="V11" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Changed — live accounts no longer hold System Manager; promising, confirm with provisioned account</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="V14" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present — 264 ignore_permissions sites in-scope, not reduced</t>
         </is>
       </c>
       <c r="W14" s="7" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="V16" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present — typo at both sites in current source (2026-10-08 re-test)</t>
         </is>
       </c>
       <c r="W16" s="7" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="V17" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Changed — tied to WC-073; systemic bypass pattern still present in source</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="V38" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present on api-dev 2026-10-08</t>
         </is>
       </c>
       <c r="W38" s="7" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="V43" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Fixed — verified in source 2026-10-08 (console.log removed from all five apps)</t>
         </is>
       </c>
       <c r="W43" s="7" t="inlineStr"/>
@@ -6401,7 +6401,7 @@
       </c>
       <c r="V51" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present on api-dev 2026-10-08</t>
         </is>
       </c>
       <c r="W51" s="7" t="inlineStr">
@@ -6509,7 +6509,7 @@
       </c>
       <c r="V52" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present on api-dev — fix may be in source but not deployed</t>
         </is>
       </c>
       <c r="W52" s="7" t="inlineStr">
@@ -9118,7 +9118,7 @@
       </c>
       <c r="V77" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Fixed — hardcoded key removed; rotate the committed keys (still in git history)</t>
         </is>
       </c>
       <c r="W77" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Retest #2 (2026-10-20): verify client fixes, add retest report and remediation plan
Independent retest against current dev source and live api-dev, plus runtime
confirmation of the two write-side S1s on the isolated stack:
- WC-084 still present (East/West account closed a North batch end to end)
- WC-095 fixed for non-System-Manager accounts (403 refusal), conditional on
  account role since the centre check exempts System Manager
- WC-011, WC-130 fixed; WC-131/129/068/073/133/134 partial; WC-088/079/105/128/
  013/004 and the live-config items still present (WC-128 corrects an earlier note)

Adds docs/retest-report and docs/remediation-plan (7 workstreams, all 87 findings);
updates the register (WC-138) and the tracker Today's Status.
</commit_message>
<xml_diff>
--- a/tracker/WeConnect-QA-Bug-Tracker.xlsx
+++ b/tracker/WeConnect-QA-Bug-Tracker.xlsx
@@ -1198,7 +1198,7 @@
       </c>
       <c r="V2" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
         </is>
       </c>
       <c r="W2" s="7" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="V3" s="9" t="inlineStr">
         <is>
-          <t>Still present — close_batch has no centre/permission check in current source</t>
+          <t>Still present — RUNTIME CONFIRMED 2026-10-20: East/West account closed a North batch ('Batch closed successfully'); no centre check in close_batch</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="V4" s="9" t="inlineStr">
         <is>
-          <t>Possibly fixed — new centre-scope layer in invoice.py; unconfirmed (write path, SP account not provisioned)</t>
+          <t>Fixed for non-System-Manager accounts — RUNTIME CONFIRMED 2026-10-20: non-SM East/West account raising a North invoice refused with HTTP 403; breaches only for System Manager accounts (live accounts are non-SM)</t>
         </is>
       </c>
       <c r="W4" s="7" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="V6" s="9" t="inlineStr">
         <is>
-          <t>Still present on api-dev 2026-10-08</t>
+          <t>Still present on api-dev — Python traceback in error body</t>
         </is>
       </c>
       <c r="W6" s="7" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="V7" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="V10" s="9" t="inlineStr">
         <is>
-          <t>Partially fixed — youth_skilling specs now require auth; batch_management spec still public</t>
+          <t>Partially fixed — youth_skilling specs now require auth; batch_management swagger_spec still public</t>
         </is>
       </c>
       <c r="W10" s="7" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="V11" s="9" t="inlineStr">
         <is>
-          <t>Changed — live accounts no longer hold System Manager; promising, confirm with provisioned account</t>
+          <t>Partially fixed — accounts no longer hold System Manager (live); source ignore_permissions bypass unchanged</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="V13" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="V14" s="9" t="inlineStr">
         <is>
-          <t>Still present — 264 ignore_permissions sites in-scope, not reduced</t>
+          <t>Still present — 322 ignore_permissions sites (up from ~296)</t>
         </is>
       </c>
       <c r="W14" s="7" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="V15" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
         </is>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="V16" s="9" t="inlineStr">
         <is>
-          <t>Still present — typo at both sites in current source (2026-10-08 re-test)</t>
+          <t>Still present — id=json.loads(id) typo at both sites</t>
         </is>
       </c>
       <c r="W16" s="7" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="V17" s="9" t="inlineStr">
         <is>
-          <t>Changed — tied to WC-073; systemic bypass pattern still present in source</t>
+          <t>Still present — 66 System Manager references in backend code</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="V18" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
         </is>
       </c>
       <c r="W18" s="7" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="V19" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Partially fixed — OTP now CSPRNG (secrets.randbelow); still 4-digit</t>
         </is>
       </c>
       <c r="W19" s="7" t="inlineStr"/>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="V21" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Fixed (retest 2026-10-20) — auth guard now derived from credentials, not hardcoded true</t>
         </is>
       </c>
       <c r="W21" s="7" t="inlineStr"/>
@@ -3355,7 +3355,7 @@
       </c>
       <c r="V22" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present — api_secret still written to localStorage (15 sites)</t>
         </is>
       </c>
       <c r="W22" s="7" t="inlineStr"/>
@@ -5030,7 +5030,7 @@
       </c>
       <c r="V38" s="9" t="inlineStr">
         <is>
-          <t>Still present on api-dev 2026-10-08</t>
+          <t>Still present on api-dev — no security headers</t>
         </is>
       </c>
       <c r="W38" s="7" t="inlineStr">
@@ -5241,7 +5241,7 @@
       </c>
       <c r="V40" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
         </is>
       </c>
       <c r="W40" s="7" t="inlineStr">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="V41" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
         </is>
       </c>
       <c r="W41" s="7" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="V42" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
         </is>
       </c>
       <c r="W42" s="7" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="V43" s="9" t="inlineStr">
         <is>
-          <t>Fixed — verified in source 2026-10-08 (console.log removed from all five apps)</t>
+          <t>Still present — reset OTP still logged to console (forget-password-api/store); corrects earlier 'fixed'</t>
         </is>
       </c>
       <c r="W43" s="7" t="inlineStr"/>
@@ -5674,7 +5674,7 @@
       </c>
       <c r="V44" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Partially fixed — error boundary now in 2 of 9 apps; 7 still lack one</t>
         </is>
       </c>
       <c r="W44" s="7" t="inlineStr"/>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="V45" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present — 19 committed .env files</t>
         </is>
       </c>
       <c r="W45" s="7" t="inlineStr"/>
@@ -6401,7 +6401,7 @@
       </c>
       <c r="V51" s="9" t="inlineStr">
         <is>
-          <t>Still present on api-dev 2026-10-08</t>
+          <t>Still present on api-dev — session Max-Age 7.1 days</t>
         </is>
       </c>
       <c r="W51" s="7" t="inlineStr">
@@ -6509,7 +6509,7 @@
       </c>
       <c r="V52" s="9" t="inlineStr">
         <is>
-          <t>Still present on api-dev — fix may be in source but not deployed</t>
+          <t>Still present on api-dev — CORS reflects any origin with credentials</t>
         </is>
       </c>
       <c r="W52" s="7" t="inlineStr">
@@ -9118,7 +9118,7 @@
       </c>
       <c r="V77" s="9" t="inlineStr">
         <is>
-          <t>Fixed — hardcoded key removed; rotate the committed keys (still in git history)</t>
+          <t>Partially fixed — source hardcode gone; key still committed in .env/.env.prod/.env.uat (rotate + purge history)</t>
         </is>
       </c>
       <c r="W77" s="7" t="inlineStr"/>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="V78" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Fixed (retest 2026-10-20) — stored-XSS sink removed; zero dangerouslySetInnerHTML</t>
         </is>
       </c>
       <c r="W78" s="7" t="inlineStr"/>
@@ -9332,7 +9332,7 @@
       </c>
       <c r="V79" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Partially fixed — 204 img without alt (was 264)</t>
         </is>
       </c>
       <c r="W79" s="7" t="inlineStr"/>
@@ -10323,6 +10323,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -14262,6 +14263,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Retest #2: full write-side probe battery on isolated stack (2026-10-20)
Re-ran the complete battery against current dev with writes enabled:
- WC-126 still present: Skilling Invoice 30/30, Skilling Batch 72/72 transitions accepted
- WC-125 still present: 5/12 contradictory values stored (capacity, percentages, cost)
- WC-123 still present: wrote another user's record (update_profile, unguarded)
- WC-089/WC-074 still present: 500 on bad input; 200 on failure
- WC-122 materially improved: 23/28 mass-assignment sites now allowlist-guarded (was ~10)
- WC-084 present, WC-095 fixed for non-System-Manager accounts (both confirmed earlier)

Updates the retest report (full runtime section), register (WC-138) and tracker.
</commit_message>
<xml_diff>
--- a/tracker/WeConnect-QA-Bug-Tracker.xlsx
+++ b/tracker/WeConnect-QA-Bug-Tracker.xlsx
@@ -5241,7 +5241,7 @@
       </c>
       <c r="V40" s="9" t="inlineStr">
         <is>
-          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
+          <t>Materially improved — RUNTIME 2026-10-20: add_interest rejects undeclared fields; 23/28 mass-assignment sites now allowlist-guarded (was ~10); 5 remain unguarded</t>
         </is>
       </c>
       <c r="W40" s="7" t="inlineStr">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="V41" s="9" t="inlineStr">
         <is>
-          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
+          <t>Still present — RUNTIME 2026-10-20: 5/12 contradictory values stored (negative/inverted capacity, 150% and -20% installment, negative cost); future DOB now rejected</t>
         </is>
       </c>
       <c r="W41" s="7" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="V42" s="9" t="inlineStr">
         <is>
-          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
+          <t>Still present — RUNTIME 2026-10-20: Skilling Invoice 30/30 and Skilling Batch 72/72 status transitions all accepted (no state machine)</t>
         </is>
       </c>
       <c r="W42" s="7" t="inlineStr">
@@ -6616,7 +6616,7 @@
       </c>
       <c r="V53" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present — RUNTIME 2026-10-20: wrote a field on another user's record (update_profile, one of 5 unguarded mass-assignment sites)</t>
         </is>
       </c>
       <c r="W53" s="7" t="inlineStr"/>
@@ -8077,7 +8077,7 @@
       </c>
       <c r="V67" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present — RUNTIME 2026-10-20: close_batch returns HTTP 200 on failure</t>
         </is>
       </c>
       <c r="W67" s="7" t="inlineStr"/>
@@ -8283,7 +8283,7 @@
       </c>
       <c r="V69" s="9" t="inlineStr">
         <is>
-          <t>Open — awaiting fix</t>
+          <t>Still present — RUNTIME 2026-10-20: create_pre_enquiry, create_enquiry, raise_invoice, create return 500 on bad input instead of 400</t>
         </is>
       </c>
       <c r="W69" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Retest #2: confirm WC-048 (fixed for non-admin) and WC-078 (still present)
WC-048 counselling read uses the same System Manager bypass / non-SM filter as the
invoice fix, so ordinary accounts are scoped; WC-078 delete_file_by_url still has
no ownership check. Register and tracker updated.
</commit_message>
<xml_diff>
--- a/tracker/WeConnect-QA-Bug-Tracker.xlsx
+++ b/tracker/WeConnect-QA-Bug-Tracker.xlsx
@@ -1198,7 +1198,7 @@
       </c>
       <c r="V2" s="9" t="inlineStr">
         <is>
-          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
+          <t>Fixed for non-System-Manager accounts — RUNTIME/source 2026-10-20: counselling list filters by User Permission for non-SM (same pattern as WC-095); System Manager bypass remains</t>
         </is>
       </c>
       <c r="W2" s="7" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="V13" s="9" t="inlineStr">
         <is>
-          <t>Runtime re-confirm in progress on isolated stack (2026-10-20)</t>
+          <t>Still present — source 2026-10-20: delete_file_by_url has no owner/permission check (files.py:463)</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">

</xml_diff>